<commit_message>
Combine Maybank and RHB into one weekly cash flow table
Q4 Weekly Cash Flow now shows a single combined statement with each
line tagged by bank, followed by the split of the closing balance by bank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141mGWEWvuV7DFAd6Wzc4uL
</commit_message>
<xml_diff>
--- a/TGFB_Q4_2026_Weekly_CashFlow_Forecast.xlsx
+++ b/TGFB_Q4_2026_Weekly_CashFlow_Forecast.xlsx
@@ -428,6 +428,36 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
+            <v>Combined</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Q4 Weekly Cash Flow'!$C$6:$P$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Q4 Weekly Cash Flow'!$C$31:$P$31</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
             <v>Maybank</v>
           </tx>
           <spPr>
@@ -450,37 +480,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Q4 Weekly Cash Flow'!$C$28:$P$28</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>Combined</v>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Q4 Weekly Cash Flow'!$C$6:$P$6</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Q4 Weekly Cash Flow'!$C$49:$P$49</f>
+              <f>'Q4 Weekly Cash Flow'!$C$39:$P$39</f>
             </numRef>
           </val>
         </ser>
@@ -542,7 +542,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>52</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -824,11 +824,11 @@
         </is>
       </c>
       <c r="B5" s="55">
-        <f>'Q4 Weekly Cash Flow'!Q10</f>
+        <f>'Q4 Weekly Cash Flow'!Q38</f>
         <v/>
       </c>
       <c r="C5" s="55">
-        <f>'Q4 Weekly Cash Flow'!Q31</f>
+        <f>'Q4 Weekly Cash Flow'!Q34</f>
         <v/>
       </c>
       <c r="D5" s="56">
@@ -882,7 +882,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="58">
-        <f>'Q4 Weekly Cash Flow'!Q33</f>
+        <f>'Q4 Weekly Cash Flow'!Q14</f>
         <v/>
       </c>
       <c r="D8" s="60">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B9" s="58">
-        <f>'Q4 Weekly Cash Flow'!Q14</f>
+        <f>'Q4 Weekly Cash Flow'!Q15</f>
         <v/>
       </c>
       <c r="C9" s="59" t="n">
@@ -918,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="58">
-        <f>'Q4 Weekly Cash Flow'!Q34</f>
+        <f>'Q4 Weekly Cash Flow'!Q16</f>
         <v/>
       </c>
       <c r="D10" s="60">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B11" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q17</f>
+        <f>-'Q4 Weekly Cash Flow'!Q19</f>
         <v/>
       </c>
       <c r="C11" s="59" t="n">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="B12" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q18</f>
+        <f>-'Q4 Weekly Cash Flow'!Q20</f>
         <v/>
       </c>
       <c r="C12" s="59" t="n">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="B13" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q19</f>
+        <f>-'Q4 Weekly Cash Flow'!Q21</f>
         <v/>
       </c>
       <c r="C13" s="59" t="n">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B14" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q20</f>
+        <f>-'Q4 Weekly Cash Flow'!Q22</f>
         <v/>
       </c>
       <c r="C14" s="59" t="n">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="B15" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q21</f>
+        <f>-'Q4 Weekly Cash Flow'!Q23</f>
         <v/>
       </c>
       <c r="C15" s="59" t="n">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="B16" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q22</f>
+        <f>-'Q4 Weekly Cash Flow'!Q24</f>
         <v/>
       </c>
       <c r="C16" s="59" t="n">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="B17" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q23</f>
+        <f>-'Q4 Weekly Cash Flow'!Q25</f>
         <v/>
       </c>
       <c r="C17" s="59" t="n">
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B18" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q24</f>
+        <f>-'Q4 Weekly Cash Flow'!Q26</f>
         <v/>
       </c>
       <c r="C18" s="59" t="n">
@@ -1080,7 +1080,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q36</f>
+        <f>-'Q4 Weekly Cash Flow'!Q27</f>
         <v/>
       </c>
       <c r="D19" s="60">
@@ -1098,7 +1098,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q37</f>
+        <f>-'Q4 Weekly Cash Flow'!Q28</f>
         <v/>
       </c>
       <c r="D20" s="60">
@@ -1113,11 +1113,11 @@
         </is>
       </c>
       <c r="B21" s="58">
-        <f>-'Q4 Weekly Cash Flow'!Q25</f>
+        <f>-'Q4 Weekly Cash Flow'!Q36</f>
         <v/>
       </c>
       <c r="C21" s="58">
-        <f>'Q4 Weekly Cash Flow'!Q39</f>
+        <f>'Q4 Weekly Cash Flow'!Q36</f>
         <v/>
       </c>
       <c r="D21" s="60">
@@ -1170,15 +1170,15 @@
         </is>
       </c>
       <c r="B24" s="64">
-        <f>ROUND(B23-'Q4 Weekly Cash Flow'!Q28,2)</f>
+        <f>ROUND(B23-'Q4 Weekly Cash Flow'!Q39,2)</f>
         <v/>
       </c>
       <c r="C24" s="64">
-        <f>ROUND(C23-'Q4 Weekly Cash Flow'!Q44,2)</f>
+        <f>ROUND(C23-'Q4 Weekly Cash Flow'!Q37,2)</f>
         <v/>
       </c>
       <c r="D24" s="64">
-        <f>ROUND(D23-'Q4 Weekly Cash Flow'!Q49,2)</f>
+        <f>ROUND(D23-'Q4 Weekly Cash Flow'!Q31,2)</f>
         <v/>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       <c r="B27" s="51" t="n"/>
       <c r="C27" s="51" t="n"/>
       <c r="D27" s="60">
-        <f>MIN('Q4 Weekly Cash Flow'!$C$49:$P$49)</f>
+        <f>MIN('Q4 Weekly Cash Flow'!$C$31:$P$31)</f>
         <v/>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       <c r="B28" s="51" t="n"/>
       <c r="C28" s="51" t="n"/>
       <c r="D28" s="67">
-        <f>INDEX('Q4 Weekly Cash Flow'!$C$6:$P$6,MATCH(D27,'Q4 Weekly Cash Flow'!$C$49:$P$49,0))</f>
+        <f>INDEX('Q4 Weekly Cash Flow'!$C$6:$P$6,MATCH(D27,'Q4 Weekly Cash Flow'!$C$31:$P$31,0))</f>
         <v/>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="B29" s="60">
-        <f>MIN('Q4 Weekly Cash Flow'!$C$28:$P$28)</f>
+        <f>MIN('Q4 Weekly Cash Flow'!$C$39:$P$39)</f>
         <v/>
       </c>
       <c r="C29" s="51" t="n"/>
@@ -8130,10 +8130,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q50"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="12.5" customWidth="1" min="3" max="3"/>
     <col width="12.5" customWidth="1" min="4" max="4"/>
@@ -8499,7 +8499,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="51" t="n"/>
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
       <c r="B8" s="51" t="n"/>
       <c r="C8" s="51" t="n"/>
       <c r="D8" s="51" t="n"/>
@@ -8520,7 +8524,7 @@
     <row r="9">
       <c r="A9" s="65" t="inlineStr">
         <is>
-          <t>MAYBANK</t>
+          <t>COMBINED CASH FLOW — MAYBANK + RHB</t>
         </is>
       </c>
       <c r="B9" s="66" t="n"/>
@@ -8544,63 +8548,63 @@
       <c r="A10" s="51" t="n"/>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>Opening balance</t>
+          <t>Opening balance (Maybank + RHB)</t>
         </is>
       </c>
       <c r="C10" s="56">
-        <f>'Q4 Assumptions'!B7</f>
+        <f>'Q4 Assumptions'!B7+'Q4 Assumptions'!B8</f>
         <v/>
       </c>
       <c r="D10" s="56">
-        <f>C28</f>
+        <f>C31</f>
         <v/>
       </c>
       <c r="E10" s="56">
-        <f>D28</f>
+        <f>D31</f>
         <v/>
       </c>
       <c r="F10" s="56">
-        <f>E28</f>
+        <f>E31</f>
         <v/>
       </c>
       <c r="G10" s="56">
-        <f>F28</f>
+        <f>F31</f>
         <v/>
       </c>
       <c r="H10" s="56">
-        <f>G28</f>
+        <f>G31</f>
         <v/>
       </c>
       <c r="I10" s="56">
-        <f>H28</f>
+        <f>H31</f>
         <v/>
       </c>
       <c r="J10" s="56">
-        <f>I28</f>
+        <f>I31</f>
         <v/>
       </c>
       <c r="K10" s="56">
-        <f>J28</f>
+        <f>J31</f>
         <v/>
       </c>
       <c r="L10" s="56">
-        <f>K28</f>
+        <f>K31</f>
         <v/>
       </c>
       <c r="M10" s="56">
-        <f>L28</f>
+        <f>L31</f>
         <v/>
       </c>
       <c r="N10" s="56">
-        <f>M28</f>
+        <f>M31</f>
         <v/>
       </c>
       <c r="O10" s="56">
-        <f>N28</f>
+        <f>N31</f>
         <v/>
       </c>
       <c r="P10" s="56">
-        <f>O28</f>
+        <f>O31</f>
         <v/>
       </c>
       <c r="Q10" s="86">
@@ -8632,7 +8636,11 @@
       <c r="Q11" s="51" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="51" t="n"/>
+      <c r="A12" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B12" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">   Sales — existing 34 outlets (Sep run-rate)</t>
@@ -8700,7 +8708,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="51" t="n"/>
+      <c r="A13" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B13" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">   Sales — new outlets (RM8k/day from GO)</t>
@@ -8768,66 +8780,70 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="51" t="n"/>
+      <c r="A14" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
       <c r="B14" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Investor funds</t>
+          <t xml:space="preserve">   Cash deposits (Sep daily average)</t>
         </is>
       </c>
       <c r="C14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>'Q4 Assumptions'!$B$36*C$7</f>
         <v/>
       </c>
       <c r="D14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>'Q4 Assumptions'!$B$36*D$7</f>
         <v/>
       </c>
       <c r="E14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>'Q4 Assumptions'!$B$36*E$7</f>
         <v/>
       </c>
       <c r="F14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>'Q4 Assumptions'!$B$36*F$7</f>
         <v/>
       </c>
       <c r="G14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>'Q4 Assumptions'!$B$36*G$7</f>
         <v/>
       </c>
       <c r="H14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>'Q4 Assumptions'!$B$36*H$7</f>
         <v/>
       </c>
       <c r="I14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>'Q4 Assumptions'!$B$36*I$7</f>
         <v/>
       </c>
       <c r="J14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>'Q4 Assumptions'!$B$36*J$7</f>
         <v/>
       </c>
       <c r="K14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>'Q4 Assumptions'!$B$36*K$7</f>
         <v/>
       </c>
       <c r="L14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>'Q4 Assumptions'!$B$36*L$7</f>
         <v/>
       </c>
       <c r="M14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>'Q4 Assumptions'!$B$36*M$7</f>
         <v/>
       </c>
       <c r="N14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>'Q4 Assumptions'!$B$36*N$7</f>
         <v/>
       </c>
       <c r="O14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>'Q4 Assumptions'!$B$36*O$7</f>
         <v/>
       </c>
       <c r="P14" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>'Q4 Assumptions'!$B$36*P$7</f>
         <v/>
       </c>
       <c r="Q14" s="86">
@@ -8836,293 +8852,305 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="51" t="n"/>
-      <c r="B15" s="54" t="inlineStr">
-        <is>
-          <t>Total cash in</t>
-        </is>
-      </c>
-      <c r="C15" s="61">
-        <f>SUM(C12:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="61">
-        <f>SUM(D12:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="61">
-        <f>SUM(E12:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="61">
-        <f>SUM(F12:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="61">
-        <f>SUM(G12:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="61">
-        <f>SUM(H12:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="61">
-        <f>SUM(I12:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="61">
-        <f>SUM(J12:J14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="61">
-        <f>SUM(K12:K14)</f>
-        <v/>
-      </c>
-      <c r="L15" s="61">
-        <f>SUM(L12:L14)</f>
-        <v/>
-      </c>
-      <c r="M15" s="61">
-        <f>SUM(M12:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="61">
-        <f>SUM(N12:N14)</f>
-        <v/>
-      </c>
-      <c r="O15" s="61">
-        <f>SUM(O12:O14)</f>
-        <v/>
-      </c>
-      <c r="P15" s="61">
-        <f>SUM(P12:P14)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="95">
+      <c r="A15" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
+      <c r="B15" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Investor funds</t>
+        </is>
+      </c>
+      <c r="C15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <v/>
+      </c>
+      <c r="D15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <v/>
+      </c>
+      <c r="E15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <v/>
+      </c>
+      <c r="F15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <v/>
+      </c>
+      <c r="G15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <v/>
+      </c>
+      <c r="H15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <v/>
+      </c>
+      <c r="I15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <v/>
+      </c>
+      <c r="J15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <v/>
+      </c>
+      <c r="K15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <v/>
+      </c>
+      <c r="L15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <v/>
+      </c>
+      <c r="M15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <v/>
+      </c>
+      <c r="N15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <v/>
+      </c>
+      <c r="O15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <v/>
+      </c>
+      <c r="P15" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Investor",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="86">
         <f>SUM(C15:P15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="51" t="n"/>
-      <c r="B16" s="54" t="inlineStr">
-        <is>
-          <t>Cash out</t>
-        </is>
-      </c>
-      <c r="C16" s="51" t="n"/>
-      <c r="D16" s="51" t="n"/>
-      <c r="E16" s="51" t="n"/>
-      <c r="F16" s="51" t="n"/>
-      <c r="G16" s="51" t="n"/>
-      <c r="H16" s="51" t="n"/>
-      <c r="I16" s="51" t="n"/>
-      <c r="J16" s="51" t="n"/>
-      <c r="K16" s="51" t="n"/>
-      <c r="L16" s="51" t="n"/>
-      <c r="M16" s="51" t="n"/>
-      <c r="N16" s="51" t="n"/>
-      <c r="O16" s="51" t="n"/>
-      <c r="P16" s="51" t="n"/>
-      <c r="Q16" s="51" t="n"/>
+      <c r="A16" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
+      <c r="B16" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Licensing package — Petaling Jaya balance</t>
+        </is>
+      </c>
+      <c r="C16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <v/>
+      </c>
+      <c r="D16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <v/>
+      </c>
+      <c r="E16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <v/>
+      </c>
+      <c r="F16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <v/>
+      </c>
+      <c r="G16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <v/>
+      </c>
+      <c r="H16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <v/>
+      </c>
+      <c r="I16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <v/>
+      </c>
+      <c r="J16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <v/>
+      </c>
+      <c r="K16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <v/>
+      </c>
+      <c r="L16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <v/>
+      </c>
+      <c r="M16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <v/>
+      </c>
+      <c r="N16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <v/>
+      </c>
+      <c r="O16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <v/>
+      </c>
+      <c r="P16" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="86">
+        <f>SUM(C16:P16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="51" t="n"/>
-      <c r="B17" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Operating costs — existing 34 outlets (Sep run-rate)</t>
-        </is>
-      </c>
-      <c r="C17" s="60">
-        <f>'Q4 Assumptions'!$B$33*C$7</f>
-        <v/>
-      </c>
-      <c r="D17" s="60">
-        <f>'Q4 Assumptions'!$B$33*D$7</f>
-        <v/>
-      </c>
-      <c r="E17" s="60">
-        <f>'Q4 Assumptions'!$B$33*E$7</f>
-        <v/>
-      </c>
-      <c r="F17" s="60">
-        <f>'Q4 Assumptions'!$B$33*F$7</f>
-        <v/>
-      </c>
-      <c r="G17" s="60">
-        <f>'Q4 Assumptions'!$B$33*G$7</f>
-        <v/>
-      </c>
-      <c r="H17" s="60">
-        <f>'Q4 Assumptions'!$B$33*H$7</f>
-        <v/>
-      </c>
-      <c r="I17" s="60">
-        <f>'Q4 Assumptions'!$B$33*I$7</f>
-        <v/>
-      </c>
-      <c r="J17" s="60">
-        <f>'Q4 Assumptions'!$B$33*J$7</f>
-        <v/>
-      </c>
-      <c r="K17" s="60">
-        <f>'Q4 Assumptions'!$B$33*K$7</f>
-        <v/>
-      </c>
-      <c r="L17" s="60">
-        <f>'Q4 Assumptions'!$B$33*L$7</f>
-        <v/>
-      </c>
-      <c r="M17" s="60">
-        <f>'Q4 Assumptions'!$B$33*M$7</f>
-        <v/>
-      </c>
-      <c r="N17" s="60">
-        <f>'Q4 Assumptions'!$B$33*N$7</f>
-        <v/>
-      </c>
-      <c r="O17" s="60">
-        <f>'Q4 Assumptions'!$B$33*O$7</f>
-        <v/>
-      </c>
-      <c r="P17" s="60">
-        <f>'Q4 Assumptions'!$B$33*P$7</f>
-        <v/>
-      </c>
-      <c r="Q17" s="86">
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t>Total cash in</t>
+        </is>
+      </c>
+      <c r="C17" s="61">
+        <f>SUM(C12:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="61">
+        <f>SUM(D12:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="61">
+        <f>SUM(E12:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="61">
+        <f>SUM(F12:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="61">
+        <f>SUM(G12:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="61">
+        <f>SUM(H12:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="61">
+        <f>SUM(I12:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="61">
+        <f>SUM(J12:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="61">
+        <f>SUM(K12:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="61">
+        <f>SUM(L12:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="61">
+        <f>SUM(M12:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="61">
+        <f>SUM(N12:N16)</f>
+        <v/>
+      </c>
+      <c r="O17" s="61">
+        <f>SUM(O12:O16)</f>
+        <v/>
+      </c>
+      <c r="P17" s="61">
+        <f>SUM(P12:P16)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="95">
         <f>SUM(C17:P17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="51" t="n"/>
-      <c r="B18" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Running cost new outlets — wages &amp; rental (15% of sales)</t>
-        </is>
-      </c>
-      <c r="C18" s="60">
-        <f>C13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="D18" s="60">
-        <f>D13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="E18" s="60">
-        <f>E13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="F18" s="60">
-        <f>F13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="G18" s="60">
-        <f>G13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="H18" s="60">
-        <f>H13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="I18" s="60">
-        <f>I13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="J18" s="60">
-        <f>J13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="K18" s="60">
-        <f>K13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="L18" s="60">
-        <f>L13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="M18" s="60">
-        <f>M13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="N18" s="60">
-        <f>N13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="O18" s="60">
-        <f>O13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="P18" s="60">
-        <f>P13*'Q4 Assumptions'!$B$14</f>
-        <v/>
-      </c>
-      <c r="Q18" s="86">
-        <f>SUM(C18:P18)</f>
-        <v/>
-      </c>
+      <c r="B18" s="54" t="inlineStr">
+        <is>
+          <t>Cash out</t>
+        </is>
+      </c>
+      <c r="C18" s="51" t="n"/>
+      <c r="D18" s="51" t="n"/>
+      <c r="E18" s="51" t="n"/>
+      <c r="F18" s="51" t="n"/>
+      <c r="G18" s="51" t="n"/>
+      <c r="H18" s="51" t="n"/>
+      <c r="I18" s="51" t="n"/>
+      <c r="J18" s="51" t="n"/>
+      <c r="K18" s="51" t="n"/>
+      <c r="L18" s="51" t="n"/>
+      <c r="M18" s="51" t="n"/>
+      <c r="N18" s="51" t="n"/>
+      <c r="O18" s="51" t="n"/>
+      <c r="P18" s="51" t="n"/>
+      <c r="Q18" s="51" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="51" t="n"/>
+      <c r="A19" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B19" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Capex — new outlets</t>
+          <t xml:space="preserve">   Operating costs — existing 34 outlets (Sep run-rate)</t>
         </is>
       </c>
       <c r="C19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;C$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;C$6)</f>
+        <f>'Q4 Assumptions'!$B$33*C$7</f>
         <v/>
       </c>
       <c r="D19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;D$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;D$6)</f>
+        <f>'Q4 Assumptions'!$B$33*D$7</f>
         <v/>
       </c>
       <c r="E19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;E$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;E$6)</f>
+        <f>'Q4 Assumptions'!$B$33*E$7</f>
         <v/>
       </c>
       <c r="F19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;F$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;F$6)</f>
+        <f>'Q4 Assumptions'!$B$33*F$7</f>
         <v/>
       </c>
       <c r="G19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;G$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;G$6)</f>
+        <f>'Q4 Assumptions'!$B$33*G$7</f>
         <v/>
       </c>
       <c r="H19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;H$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;H$6)</f>
+        <f>'Q4 Assumptions'!$B$33*H$7</f>
         <v/>
       </c>
       <c r="I19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;I$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;I$6)</f>
+        <f>'Q4 Assumptions'!$B$33*I$7</f>
         <v/>
       </c>
       <c r="J19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;J$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;J$6)</f>
+        <f>'Q4 Assumptions'!$B$33*J$7</f>
         <v/>
       </c>
       <c r="K19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;K$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;K$6)</f>
+        <f>'Q4 Assumptions'!$B$33*K$7</f>
         <v/>
       </c>
       <c r="L19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;L$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;L$6)</f>
+        <f>'Q4 Assumptions'!$B$33*L$7</f>
         <v/>
       </c>
       <c r="M19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;M$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;M$6)</f>
+        <f>'Q4 Assumptions'!$B$33*M$7</f>
         <v/>
       </c>
       <c r="N19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;N$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;N$6)</f>
+        <f>'Q4 Assumptions'!$B$33*N$7</f>
         <v/>
       </c>
       <c r="O19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;O$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;O$6)</f>
+        <f>'Q4 Assumptions'!$B$33*O$7</f>
         <v/>
       </c>
       <c r="P19" s="60">
-        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;P$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;P$6)</f>
+        <f>'Q4 Assumptions'!$B$33*P$7</f>
         <v/>
       </c>
       <c r="Q19" s="86">
@@ -9131,66 +9159,70 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="51" t="n"/>
+      <c r="A20" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B20" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Deposits — 5 new outlets</t>
+          <t xml:space="preserve">   Running cost new outlets — wages &amp; rental (15% of sales)</t>
         </is>
       </c>
       <c r="C20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>C13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="D20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>D13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="E20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>E13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="F20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>F13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="G20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>G13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="H20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>H13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="I20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>I13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="J20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>J13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="K20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>K13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="L20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>L13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="M20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>M13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="N20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>N13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="O20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>O13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="P20" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>P13*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="Q20" s="86">
@@ -9199,66 +9231,70 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="51" t="n"/>
+      <c r="A21" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B21" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Foreign worker expense</t>
+          <t xml:space="preserve">   Capex — new outlets</t>
         </is>
       </c>
       <c r="C21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;C$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;C$6)</f>
         <v/>
       </c>
       <c r="D21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;D$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;D$6)</f>
         <v/>
       </c>
       <c r="E21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;E$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;E$6)</f>
         <v/>
       </c>
       <c r="F21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;F$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;F$6)</f>
         <v/>
       </c>
       <c r="G21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;G$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;G$6)</f>
         <v/>
       </c>
       <c r="H21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;H$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;H$6)</f>
         <v/>
       </c>
       <c r="I21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;I$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;I$6)</f>
         <v/>
       </c>
       <c r="J21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;J$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;J$6)</f>
         <v/>
       </c>
       <c r="K21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;K$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;K$6)</f>
         <v/>
       </c>
       <c r="L21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;L$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;L$6)</f>
         <v/>
       </c>
       <c r="M21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;M$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;M$6)</f>
         <v/>
       </c>
       <c r="N21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;N$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;N$6)</f>
         <v/>
       </c>
       <c r="O21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;O$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;O$6)</f>
         <v/>
       </c>
       <c r="P21" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;P$5,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q21" s="86">
@@ -9267,66 +9303,70 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="51" t="n"/>
+      <c r="A22" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B22" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Investment — Bebeks</t>
+          <t xml:space="preserve">   Deposits — 5 new outlets</t>
         </is>
       </c>
       <c r="C22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
         <v/>
       </c>
       <c r="D22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
         <v/>
       </c>
       <c r="E22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
         <v/>
       </c>
       <c r="F22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
         <v/>
       </c>
       <c r="G22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
         <v/>
       </c>
       <c r="H22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
         <v/>
       </c>
       <c r="I22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
         <v/>
       </c>
       <c r="J22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
         <v/>
       </c>
       <c r="K22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
         <v/>
       </c>
       <c r="L22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
         <v/>
       </c>
       <c r="M22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
         <v/>
       </c>
       <c r="N22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
         <v/>
       </c>
       <c r="O22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
         <v/>
       </c>
       <c r="P22" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Deposit",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q22" s="86">
@@ -9335,66 +9375,70 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="51" t="n"/>
+      <c r="A23" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B23" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Investment — Kopitiam</t>
+          <t xml:space="preserve">   Foreign worker expense</t>
         </is>
       </c>
       <c r="C23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
         <v/>
       </c>
       <c r="D23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
         <v/>
       </c>
       <c r="E23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
         <v/>
       </c>
       <c r="F23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
         <v/>
       </c>
       <c r="G23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
         <v/>
       </c>
       <c r="H23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
         <v/>
       </c>
       <c r="I23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
         <v/>
       </c>
       <c r="J23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
         <v/>
       </c>
       <c r="K23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
         <v/>
       </c>
       <c r="L23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
         <v/>
       </c>
       <c r="M23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
         <v/>
       </c>
       <c r="N23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
         <v/>
       </c>
       <c r="O23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
         <v/>
       </c>
       <c r="P23" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Foreign worker",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q23" s="86">
@@ -9403,66 +9447,70 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="51" t="n"/>
+      <c r="A24" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B24" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   SST Sep–Oct</t>
+          <t xml:space="preserve">   Investment — Bebeks</t>
         </is>
       </c>
       <c r="C24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
         <v/>
       </c>
       <c r="D24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
         <v/>
       </c>
       <c r="E24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
         <v/>
       </c>
       <c r="F24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
         <v/>
       </c>
       <c r="G24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
         <v/>
       </c>
       <c r="H24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
         <v/>
       </c>
       <c r="I24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
         <v/>
       </c>
       <c r="J24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
         <v/>
       </c>
       <c r="K24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
         <v/>
       </c>
       <c r="L24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
         <v/>
       </c>
       <c r="M24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
         <v/>
       </c>
       <c r="N24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
         <v/>
       </c>
       <c r="O24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
         <v/>
       </c>
       <c r="P24" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bebeks",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q24" s="86">
@@ -9471,66 +9519,70 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="51" t="n"/>
+      <c r="A25" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
       <c r="B25" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Transfer to RHB (payroll funding)</t>
+          <t xml:space="preserve">   Investment — Kopitiam</t>
         </is>
       </c>
       <c r="C25" s="60">
-        <f>C39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
         <v/>
       </c>
       <c r="D25" s="60">
-        <f>D39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
         <v/>
       </c>
       <c r="E25" s="60">
-        <f>E39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
         <v/>
       </c>
       <c r="F25" s="60">
-        <f>F39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
         <v/>
       </c>
       <c r="G25" s="60">
-        <f>G39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
         <v/>
       </c>
       <c r="H25" s="60">
-        <f>H39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
         <v/>
       </c>
       <c r="I25" s="60">
-        <f>I39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
         <v/>
       </c>
       <c r="J25" s="60">
-        <f>J39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
         <v/>
       </c>
       <c r="K25" s="60">
-        <f>K39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
         <v/>
       </c>
       <c r="L25" s="60">
-        <f>L39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
         <v/>
       </c>
       <c r="M25" s="60">
-        <f>M39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
         <v/>
       </c>
       <c r="N25" s="60">
-        <f>N39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
         <v/>
       </c>
       <c r="O25" s="60">
-        <f>O39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
         <v/>
       </c>
       <c r="P25" s="60">
-        <f>P39</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Kopitiam",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q25" s="86">
@@ -9539,134 +9591,142 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="51" t="n"/>
-      <c r="B26" s="54" t="inlineStr">
-        <is>
-          <t>Total cash out</t>
-        </is>
-      </c>
-      <c r="C26" s="61">
-        <f>SUM(C17:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="61">
-        <f>SUM(D17:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="61">
-        <f>SUM(E17:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="61">
-        <f>SUM(F17:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="61">
-        <f>SUM(G17:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="61">
-        <f>SUM(H17:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="61">
-        <f>SUM(I17:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="61">
-        <f>SUM(J17:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="61">
-        <f>SUM(K17:K25)</f>
-        <v/>
-      </c>
-      <c r="L26" s="61">
-        <f>SUM(L17:L25)</f>
-        <v/>
-      </c>
-      <c r="M26" s="61">
-        <f>SUM(M17:M25)</f>
-        <v/>
-      </c>
-      <c r="N26" s="61">
-        <f>SUM(N17:N25)</f>
-        <v/>
-      </c>
-      <c r="O26" s="61">
-        <f>SUM(O17:O25)</f>
-        <v/>
-      </c>
-      <c r="P26" s="61">
-        <f>SUM(P17:P25)</f>
-        <v/>
-      </c>
-      <c r="Q26" s="95">
+      <c r="A26" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
+      <c r="B26" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SST Sep–Oct</t>
+        </is>
+      </c>
+      <c r="C26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <v/>
+      </c>
+      <c r="D26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <v/>
+      </c>
+      <c r="E26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <v/>
+      </c>
+      <c r="F26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <v/>
+      </c>
+      <c r="G26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <v/>
+      </c>
+      <c r="H26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <v/>
+      </c>
+      <c r="I26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <v/>
+      </c>
+      <c r="J26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <v/>
+      </c>
+      <c r="K26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <v/>
+      </c>
+      <c r="L26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <v/>
+      </c>
+      <c r="M26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <v/>
+      </c>
+      <c r="N26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <v/>
+      </c>
+      <c r="O26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <v/>
+      </c>
+      <c r="P26" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"SST",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="86">
         <f>SUM(C26:P26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="51" t="n"/>
-      <c r="B27" s="54" t="inlineStr">
-        <is>
-          <t>Net cash flow</t>
-        </is>
-      </c>
-      <c r="C27" s="56">
-        <f>C15-C26</f>
-        <v/>
-      </c>
-      <c r="D27" s="56">
-        <f>D15-D26</f>
-        <v/>
-      </c>
-      <c r="E27" s="56">
-        <f>E15-E26</f>
-        <v/>
-      </c>
-      <c r="F27" s="56">
-        <f>F15-F26</f>
-        <v/>
-      </c>
-      <c r="G27" s="56">
-        <f>G15-G26</f>
-        <v/>
-      </c>
-      <c r="H27" s="56">
-        <f>H15-H26</f>
-        <v/>
-      </c>
-      <c r="I27" s="56">
-        <f>I15-I26</f>
-        <v/>
-      </c>
-      <c r="J27" s="56">
-        <f>J15-J26</f>
-        <v/>
-      </c>
-      <c r="K27" s="56">
-        <f>K15-K26</f>
-        <v/>
-      </c>
-      <c r="L27" s="56">
-        <f>L15-L26</f>
-        <v/>
-      </c>
-      <c r="M27" s="56">
-        <f>M15-M26</f>
-        <v/>
-      </c>
-      <c r="N27" s="56">
-        <f>N15-N26</f>
-        <v/>
-      </c>
-      <c r="O27" s="56">
-        <f>O15-O26</f>
-        <v/>
-      </c>
-      <c r="P27" s="56">
-        <f>P15-P26</f>
+      <c r="A27" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
+      <c r="B27" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Payroll (25th)</t>
+        </is>
+      </c>
+      <c r="C27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <v/>
+      </c>
+      <c r="D27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <v/>
+      </c>
+      <c r="E27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <v/>
+      </c>
+      <c r="F27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <v/>
+      </c>
+      <c r="G27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <v/>
+      </c>
+      <c r="H27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <v/>
+      </c>
+      <c r="I27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <v/>
+      </c>
+      <c r="J27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <v/>
+      </c>
+      <c r="K27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <v/>
+      </c>
+      <c r="L27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <v/>
+      </c>
+      <c r="M27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <v/>
+      </c>
+      <c r="N27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <v/>
+      </c>
+      <c r="O27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <v/>
+      </c>
+      <c r="P27" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q27" s="86">
@@ -9675,190 +9735,284 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="51" t="n"/>
-      <c r="B28" s="96" t="inlineStr">
-        <is>
-          <t>Closing balance — Maybank</t>
-        </is>
-      </c>
-      <c r="C28" s="86">
-        <f>C10+C27</f>
-        <v/>
-      </c>
-      <c r="D28" s="86">
-        <f>D10+D27</f>
-        <v/>
-      </c>
-      <c r="E28" s="86">
-        <f>E10+E27</f>
-        <v/>
-      </c>
-      <c r="F28" s="86">
-        <f>F10+F27</f>
-        <v/>
-      </c>
-      <c r="G28" s="86">
-        <f>G10+G27</f>
-        <v/>
-      </c>
-      <c r="H28" s="86">
-        <f>H10+H27</f>
-        <v/>
-      </c>
-      <c r="I28" s="86">
-        <f>I10+I27</f>
-        <v/>
-      </c>
-      <c r="J28" s="86">
-        <f>J10+J27</f>
-        <v/>
-      </c>
-      <c r="K28" s="86">
-        <f>K10+K27</f>
-        <v/>
-      </c>
-      <c r="L28" s="86">
-        <f>L10+L27</f>
-        <v/>
-      </c>
-      <c r="M28" s="86">
-        <f>M10+M27</f>
-        <v/>
-      </c>
-      <c r="N28" s="86">
-        <f>N10+N27</f>
-        <v/>
-      </c>
-      <c r="O28" s="86">
-        <f>O10+O27</f>
-        <v/>
-      </c>
-      <c r="P28" s="86">
-        <f>P10+P27</f>
+      <c r="A28" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
+      <c r="B28" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Staff bonus</t>
+        </is>
+      </c>
+      <c r="C28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <v/>
+      </c>
+      <c r="D28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <v/>
+      </c>
+      <c r="E28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <v/>
+      </c>
+      <c r="F28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <v/>
+      </c>
+      <c r="G28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <v/>
+      </c>
+      <c r="H28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <v/>
+      </c>
+      <c r="I28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <v/>
+      </c>
+      <c r="J28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <v/>
+      </c>
+      <c r="K28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <v/>
+      </c>
+      <c r="L28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <v/>
+      </c>
+      <c r="M28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <v/>
+      </c>
+      <c r="N28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <v/>
+      </c>
+      <c r="O28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <v/>
+      </c>
+      <c r="P28" s="60">
+        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
         <v/>
       </c>
       <c r="Q28" s="86">
-        <f>P28</f>
+        <f>SUM(C28:P28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="51" t="n"/>
-      <c r="B29" s="51" t="n"/>
-      <c r="C29" s="51" t="n"/>
-      <c r="D29" s="51" t="n"/>
-      <c r="E29" s="51" t="n"/>
-      <c r="F29" s="51" t="n"/>
-      <c r="G29" s="51" t="n"/>
-      <c r="H29" s="51" t="n"/>
-      <c r="I29" s="51" t="n"/>
-      <c r="J29" s="51" t="n"/>
-      <c r="K29" s="51" t="n"/>
-      <c r="L29" s="51" t="n"/>
-      <c r="M29" s="51" t="n"/>
-      <c r="N29" s="51" t="n"/>
-      <c r="O29" s="51" t="n"/>
-      <c r="P29" s="51" t="n"/>
-      <c r="Q29" s="51" t="n"/>
+      <c r="B29" s="54" t="inlineStr">
+        <is>
+          <t>Total cash out</t>
+        </is>
+      </c>
+      <c r="C29" s="61">
+        <f>SUM(C19:C28)</f>
+        <v/>
+      </c>
+      <c r="D29" s="61">
+        <f>SUM(D19:D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="61">
+        <f>SUM(E19:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="61">
+        <f>SUM(F19:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="61">
+        <f>SUM(G19:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="61">
+        <f>SUM(H19:H28)</f>
+        <v/>
+      </c>
+      <c r="I29" s="61">
+        <f>SUM(I19:I28)</f>
+        <v/>
+      </c>
+      <c r="J29" s="61">
+        <f>SUM(J19:J28)</f>
+        <v/>
+      </c>
+      <c r="K29" s="61">
+        <f>SUM(K19:K28)</f>
+        <v/>
+      </c>
+      <c r="L29" s="61">
+        <f>SUM(L19:L28)</f>
+        <v/>
+      </c>
+      <c r="M29" s="61">
+        <f>SUM(M19:M28)</f>
+        <v/>
+      </c>
+      <c r="N29" s="61">
+        <f>SUM(N19:N28)</f>
+        <v/>
+      </c>
+      <c r="O29" s="61">
+        <f>SUM(O19:O28)</f>
+        <v/>
+      </c>
+      <c r="P29" s="61">
+        <f>SUM(P19:P28)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="95">
+        <f>SUM(C29:P29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="65" t="inlineStr">
-        <is>
-          <t>RHB</t>
-        </is>
-      </c>
-      <c r="B30" s="66" t="n"/>
-      <c r="C30" s="66" t="n"/>
-      <c r="D30" s="66" t="n"/>
-      <c r="E30" s="66" t="n"/>
-      <c r="F30" s="66" t="n"/>
-      <c r="G30" s="66" t="n"/>
-      <c r="H30" s="66" t="n"/>
-      <c r="I30" s="66" t="n"/>
-      <c r="J30" s="66" t="n"/>
-      <c r="K30" s="66" t="n"/>
-      <c r="L30" s="66" t="n"/>
-      <c r="M30" s="66" t="n"/>
-      <c r="N30" s="66" t="n"/>
-      <c r="O30" s="66" t="n"/>
-      <c r="P30" s="66" t="n"/>
-      <c r="Q30" s="66" t="n"/>
+      <c r="A30" s="51" t="n"/>
+      <c r="B30" s="54" t="inlineStr">
+        <is>
+          <t>Net cash flow</t>
+        </is>
+      </c>
+      <c r="C30" s="56">
+        <f>C17-C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="56">
+        <f>D17-D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="56">
+        <f>E17-E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="56">
+        <f>F17-F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="56">
+        <f>G17-G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="56">
+        <f>H17-H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="56">
+        <f>I17-I29</f>
+        <v/>
+      </c>
+      <c r="J30" s="56">
+        <f>J17-J29</f>
+        <v/>
+      </c>
+      <c r="K30" s="56">
+        <f>K17-K29</f>
+        <v/>
+      </c>
+      <c r="L30" s="56">
+        <f>L17-L29</f>
+        <v/>
+      </c>
+      <c r="M30" s="56">
+        <f>M17-M29</f>
+        <v/>
+      </c>
+      <c r="N30" s="56">
+        <f>N17-N29</f>
+        <v/>
+      </c>
+      <c r="O30" s="56">
+        <f>O17-O29</f>
+        <v/>
+      </c>
+      <c r="P30" s="56">
+        <f>P17-P29</f>
+        <v/>
+      </c>
+      <c r="Q30" s="86">
+        <f>SUM(C30:P30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="51" t="n"/>
-      <c r="B31" s="54" t="inlineStr">
-        <is>
-          <t>Opening balance</t>
-        </is>
-      </c>
-      <c r="C31" s="56">
-        <f>'Q4 Assumptions'!B8</f>
-        <v/>
-      </c>
-      <c r="D31" s="56">
-        <f>C44</f>
-        <v/>
-      </c>
-      <c r="E31" s="56">
-        <f>D44</f>
-        <v/>
-      </c>
-      <c r="F31" s="56">
-        <f>E44</f>
-        <v/>
-      </c>
-      <c r="G31" s="56">
-        <f>F44</f>
-        <v/>
-      </c>
-      <c r="H31" s="56">
-        <f>G44</f>
-        <v/>
-      </c>
-      <c r="I31" s="56">
-        <f>H44</f>
-        <v/>
-      </c>
-      <c r="J31" s="56">
-        <f>I44</f>
-        <v/>
-      </c>
-      <c r="K31" s="56">
-        <f>J44</f>
-        <v/>
-      </c>
-      <c r="L31" s="56">
-        <f>K44</f>
-        <v/>
-      </c>
-      <c r="M31" s="56">
-        <f>L44</f>
-        <v/>
-      </c>
-      <c r="N31" s="56">
-        <f>M44</f>
-        <v/>
-      </c>
-      <c r="O31" s="56">
-        <f>N44</f>
-        <v/>
-      </c>
-      <c r="P31" s="56">
-        <f>O44</f>
+      <c r="B31" s="62" t="inlineStr">
+        <is>
+          <t>Closing balance (Maybank + RHB)</t>
+        </is>
+      </c>
+      <c r="C31" s="63">
+        <f>C10+C30</f>
+        <v/>
+      </c>
+      <c r="D31" s="63">
+        <f>D10+D30</f>
+        <v/>
+      </c>
+      <c r="E31" s="63">
+        <f>E10+E30</f>
+        <v/>
+      </c>
+      <c r="F31" s="63">
+        <f>F10+F30</f>
+        <v/>
+      </c>
+      <c r="G31" s="63">
+        <f>G10+G30</f>
+        <v/>
+      </c>
+      <c r="H31" s="63">
+        <f>H10+H30</f>
+        <v/>
+      </c>
+      <c r="I31" s="63">
+        <f>I10+I30</f>
+        <v/>
+      </c>
+      <c r="J31" s="63">
+        <f>J10+J30</f>
+        <v/>
+      </c>
+      <c r="K31" s="63">
+        <f>K10+K30</f>
+        <v/>
+      </c>
+      <c r="L31" s="63">
+        <f>L10+L30</f>
+        <v/>
+      </c>
+      <c r="M31" s="63">
+        <f>M10+M30</f>
+        <v/>
+      </c>
+      <c r="N31" s="63">
+        <f>N10+N30</f>
+        <v/>
+      </c>
+      <c r="O31" s="63">
+        <f>O10+O30</f>
+        <v/>
+      </c>
+      <c r="P31" s="63">
+        <f>P10+P30</f>
         <v/>
       </c>
       <c r="Q31" s="86">
-        <f>C31</f>
+        <f>P31</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="51" t="n"/>
-      <c r="B32" s="54" t="inlineStr">
-        <is>
-          <t>Cash in</t>
-        </is>
-      </c>
+      <c r="B32" s="51" t="n"/>
       <c r="C32" s="51" t="n"/>
       <c r="D32" s="51" t="n"/>
       <c r="E32" s="51" t="n"/>
@@ -9876,225 +10030,234 @@
       <c r="Q32" s="51" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="51" t="n"/>
-      <c r="B33" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Cash deposits (Sep daily average)</t>
-        </is>
-      </c>
-      <c r="C33" s="60">
-        <f>'Q4 Assumptions'!$B$36*C$7</f>
-        <v/>
-      </c>
-      <c r="D33" s="60">
-        <f>'Q4 Assumptions'!$B$36*D$7</f>
-        <v/>
-      </c>
-      <c r="E33" s="60">
-        <f>'Q4 Assumptions'!$B$36*E$7</f>
-        <v/>
-      </c>
-      <c r="F33" s="60">
-        <f>'Q4 Assumptions'!$B$36*F$7</f>
-        <v/>
-      </c>
-      <c r="G33" s="60">
-        <f>'Q4 Assumptions'!$B$36*G$7</f>
-        <v/>
-      </c>
-      <c r="H33" s="60">
-        <f>'Q4 Assumptions'!$B$36*H$7</f>
-        <v/>
-      </c>
-      <c r="I33" s="60">
-        <f>'Q4 Assumptions'!$B$36*I$7</f>
-        <v/>
-      </c>
-      <c r="J33" s="60">
-        <f>'Q4 Assumptions'!$B$36*J$7</f>
-        <v/>
-      </c>
-      <c r="K33" s="60">
-        <f>'Q4 Assumptions'!$B$36*K$7</f>
-        <v/>
-      </c>
-      <c r="L33" s="60">
-        <f>'Q4 Assumptions'!$B$36*L$7</f>
-        <v/>
-      </c>
-      <c r="M33" s="60">
-        <f>'Q4 Assumptions'!$B$36*M$7</f>
-        <v/>
-      </c>
-      <c r="N33" s="60">
-        <f>'Q4 Assumptions'!$B$36*N$7</f>
-        <v/>
-      </c>
-      <c r="O33" s="60">
-        <f>'Q4 Assumptions'!$B$36*O$7</f>
-        <v/>
-      </c>
-      <c r="P33" s="60">
-        <f>'Q4 Assumptions'!$B$36*P$7</f>
-        <v/>
-      </c>
-      <c r="Q33" s="86">
-        <f>SUM(C33:P33)</f>
-        <v/>
-      </c>
+      <c r="A33" s="65" t="inlineStr">
+        <is>
+          <t>SPLIT OF CLOSING BALANCE BY BANK</t>
+        </is>
+      </c>
+      <c r="B33" s="66" t="n"/>
+      <c r="C33" s="66" t="n"/>
+      <c r="D33" s="66" t="n"/>
+      <c r="E33" s="66" t="n"/>
+      <c r="F33" s="66" t="n"/>
+      <c r="G33" s="66" t="n"/>
+      <c r="H33" s="66" t="n"/>
+      <c r="I33" s="66" t="n"/>
+      <c r="J33" s="66" t="n"/>
+      <c r="K33" s="66" t="n"/>
+      <c r="L33" s="66" t="n"/>
+      <c r="M33" s="66" t="n"/>
+      <c r="N33" s="66" t="n"/>
+      <c r="O33" s="66" t="n"/>
+      <c r="P33" s="66" t="n"/>
+      <c r="Q33" s="66" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="51" t="n"/>
+      <c r="A34" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
       <c r="B34" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Licensing package — Petaling Jaya balance</t>
+          <t xml:space="preserve">   RHB opening balance</t>
         </is>
       </c>
       <c r="C34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>'Q4 Assumptions'!B8</f>
         <v/>
       </c>
       <c r="D34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>C37</f>
         <v/>
       </c>
       <c r="E34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>D37</f>
         <v/>
       </c>
       <c r="F34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>E37</f>
         <v/>
       </c>
       <c r="G34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>F37</f>
         <v/>
       </c>
       <c r="H34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>G37</f>
         <v/>
       </c>
       <c r="I34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>H37</f>
         <v/>
       </c>
       <c r="J34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>I37</f>
         <v/>
       </c>
       <c r="K34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>J37</f>
         <v/>
       </c>
       <c r="L34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>K37</f>
         <v/>
       </c>
       <c r="M34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>L37</f>
         <v/>
       </c>
       <c r="N34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>M37</f>
         <v/>
       </c>
       <c r="O34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>N37</f>
         <v/>
       </c>
       <c r="P34" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Licensing",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>O37</f>
         <v/>
       </c>
       <c r="Q34" s="86">
-        <f>SUM(C34:P34)</f>
+        <f>C34</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="51" t="n"/>
-      <c r="B35" s="54" t="inlineStr">
-        <is>
-          <t>Cash out</t>
-        </is>
-      </c>
-      <c r="C35" s="51" t="n"/>
-      <c r="D35" s="51" t="n"/>
-      <c r="E35" s="51" t="n"/>
-      <c r="F35" s="51" t="n"/>
-      <c r="G35" s="51" t="n"/>
-      <c r="H35" s="51" t="n"/>
-      <c r="I35" s="51" t="n"/>
-      <c r="J35" s="51" t="n"/>
-      <c r="K35" s="51" t="n"/>
-      <c r="L35" s="51" t="n"/>
-      <c r="M35" s="51" t="n"/>
-      <c r="N35" s="51" t="n"/>
-      <c r="O35" s="51" t="n"/>
-      <c r="P35" s="51" t="n"/>
+      <c r="A35" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
+      <c r="B35" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   RHB balance before top-up</t>
+        </is>
+      </c>
+      <c r="C35" s="60">
+        <f>C34+C14+C16-C27-C28</f>
+        <v/>
+      </c>
+      <c r="D35" s="60">
+        <f>D34+D14+D16-D27-D28</f>
+        <v/>
+      </c>
+      <c r="E35" s="60">
+        <f>E34+E14+E16-E27-E28</f>
+        <v/>
+      </c>
+      <c r="F35" s="60">
+        <f>F34+F14+F16-F27-F28</f>
+        <v/>
+      </c>
+      <c r="G35" s="60">
+        <f>G34+G14+G16-G27-G28</f>
+        <v/>
+      </c>
+      <c r="H35" s="60">
+        <f>H34+H14+H16-H27-H28</f>
+        <v/>
+      </c>
+      <c r="I35" s="60">
+        <f>I34+I14+I16-I27-I28</f>
+        <v/>
+      </c>
+      <c r="J35" s="60">
+        <f>J34+J14+J16-J27-J28</f>
+        <v/>
+      </c>
+      <c r="K35" s="60">
+        <f>K34+K14+K16-K27-K28</f>
+        <v/>
+      </c>
+      <c r="L35" s="60">
+        <f>L34+L14+L16-L27-L28</f>
+        <v/>
+      </c>
+      <c r="M35" s="60">
+        <f>M34+M14+M16-M27-M28</f>
+        <v/>
+      </c>
+      <c r="N35" s="60">
+        <f>N34+N14+N16-N27-N28</f>
+        <v/>
+      </c>
+      <c r="O35" s="60">
+        <f>O34+O14+O16-O27-O28</f>
+        <v/>
+      </c>
+      <c r="P35" s="60">
+        <f>P34+P14+P16-P27-P28</f>
+        <v/>
+      </c>
       <c r="Q35" s="51" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="51" t="n"/>
+      <c r="A36" s="80" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
       <c r="B36" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Payroll (25th)</t>
+          <t xml:space="preserve">   Transfer Maybank → RHB (top-up to minimum; nets to zero combined)</t>
         </is>
       </c>
       <c r="C36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-C35)</f>
         <v/>
       </c>
       <c r="D36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-D35)</f>
         <v/>
       </c>
       <c r="E36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-E35)</f>
         <v/>
       </c>
       <c r="F36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-F35)</f>
         <v/>
       </c>
       <c r="G36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-G35)</f>
         <v/>
       </c>
       <c r="H36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-H35)</f>
         <v/>
       </c>
       <c r="I36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-I35)</f>
         <v/>
       </c>
       <c r="J36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-J35)</f>
         <v/>
       </c>
       <c r="K36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-K35)</f>
         <v/>
       </c>
       <c r="L36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-L35)</f>
         <v/>
       </c>
       <c r="M36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-M35)</f>
         <v/>
       </c>
       <c r="N36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-N35)</f>
         <v/>
       </c>
       <c r="O36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-O35)</f>
         <v/>
       </c>
       <c r="P36" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Payroll",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+        <f>MAX(0,'Q4 Assumptions'!$B$38-P35)</f>
         <v/>
       </c>
       <c r="Q36" s="86">
@@ -10103,807 +10266,285 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="51" t="n"/>
-      <c r="B37" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Staff bonus</t>
-        </is>
-      </c>
-      <c r="C37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;C$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;C$6)</f>
-        <v/>
-      </c>
-      <c r="D37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;D$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;D$6)</f>
-        <v/>
-      </c>
-      <c r="E37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;E$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;E$6)</f>
-        <v/>
-      </c>
-      <c r="F37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;F$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;F$6)</f>
-        <v/>
-      </c>
-      <c r="G37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;G$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;G$6)</f>
-        <v/>
-      </c>
-      <c r="H37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;H$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;H$6)</f>
-        <v/>
-      </c>
-      <c r="I37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;I$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;I$6)</f>
-        <v/>
-      </c>
-      <c r="J37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;J$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;J$6)</f>
-        <v/>
-      </c>
-      <c r="K37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;K$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;K$6)</f>
-        <v/>
-      </c>
-      <c r="L37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;L$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;L$6)</f>
-        <v/>
-      </c>
-      <c r="M37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;M$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;M$6)</f>
-        <v/>
-      </c>
-      <c r="N37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;N$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;N$6)</f>
-        <v/>
-      </c>
-      <c r="O37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;O$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;O$6)</f>
-        <v/>
-      </c>
-      <c r="P37" s="60">
-        <f>SUMIFS('Q4 Assumptions'!$C$42:$C$58,'Q4 Assumptions'!$D$42:$D$58,"Bonus",'Q4 Assumptions'!$B$42:$B$58,"&gt;="&amp;P$5,'Q4 Assumptions'!$B$42:$B$58,"&lt;="&amp;P$6)</f>
+      <c r="A37" s="80" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
+      <c r="B37" s="96" t="inlineStr">
+        <is>
+          <t>Closing balance — RHB</t>
+        </is>
+      </c>
+      <c r="C37" s="86">
+        <f>C35+C36</f>
+        <v/>
+      </c>
+      <c r="D37" s="86">
+        <f>D35+D36</f>
+        <v/>
+      </c>
+      <c r="E37" s="86">
+        <f>E35+E36</f>
+        <v/>
+      </c>
+      <c r="F37" s="86">
+        <f>F35+F36</f>
+        <v/>
+      </c>
+      <c r="G37" s="86">
+        <f>G35+G36</f>
+        <v/>
+      </c>
+      <c r="H37" s="86">
+        <f>H35+H36</f>
+        <v/>
+      </c>
+      <c r="I37" s="86">
+        <f>I35+I36</f>
+        <v/>
+      </c>
+      <c r="J37" s="86">
+        <f>J35+J36</f>
+        <v/>
+      </c>
+      <c r="K37" s="86">
+        <f>K35+K36</f>
+        <v/>
+      </c>
+      <c r="L37" s="86">
+        <f>L35+L36</f>
+        <v/>
+      </c>
+      <c r="M37" s="86">
+        <f>M35+M36</f>
+        <v/>
+      </c>
+      <c r="N37" s="86">
+        <f>N35+N36</f>
+        <v/>
+      </c>
+      <c r="O37" s="86">
+        <f>O35+O36</f>
+        <v/>
+      </c>
+      <c r="P37" s="86">
+        <f>P35+P36</f>
         <v/>
       </c>
       <c r="Q37" s="86">
-        <f>SUM(C37:P37)</f>
+        <f>P37</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="51" t="n"/>
-      <c r="B38" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Balance before top-up</t>
-        </is>
-      </c>
-      <c r="C38" s="64">
-        <f>C31+C33+C34-C36-C37</f>
-        <v/>
-      </c>
-      <c r="D38" s="64">
-        <f>D31+D33+D34-D36-D37</f>
-        <v/>
-      </c>
-      <c r="E38" s="64">
-        <f>E31+E33+E34-E36-E37</f>
-        <v/>
-      </c>
-      <c r="F38" s="64">
-        <f>F31+F33+F34-F36-F37</f>
-        <v/>
-      </c>
-      <c r="G38" s="64">
-        <f>G31+G33+G34-G36-G37</f>
-        <v/>
-      </c>
-      <c r="H38" s="64">
-        <f>H31+H33+H34-H36-H37</f>
-        <v/>
-      </c>
-      <c r="I38" s="64">
-        <f>I31+I33+I34-I36-I37</f>
-        <v/>
-      </c>
-      <c r="J38" s="64">
-        <f>J31+J33+J34-J36-J37</f>
-        <v/>
-      </c>
-      <c r="K38" s="64">
-        <f>K31+K33+K34-K36-K37</f>
-        <v/>
-      </c>
-      <c r="L38" s="64">
-        <f>L31+L33+L34-L36-L37</f>
-        <v/>
-      </c>
-      <c r="M38" s="64">
-        <f>M31+M33+M34-M36-M37</f>
-        <v/>
-      </c>
-      <c r="N38" s="64">
-        <f>N31+N33+N34-N36-N37</f>
-        <v/>
-      </c>
-      <c r="O38" s="64">
-        <f>O31+O33+O34-O36-O37</f>
-        <v/>
-      </c>
-      <c r="P38" s="64">
-        <f>P31+P33+P34-P36-P37</f>
-        <v/>
-      </c>
-      <c r="Q38" s="51" t="n"/>
+      <c r="A38" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
+      <c r="B38" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Maybank opening balance</t>
+        </is>
+      </c>
+      <c r="C38" s="60">
+        <f>'Q4 Assumptions'!B7</f>
+        <v/>
+      </c>
+      <c r="D38" s="60">
+        <f>C39</f>
+        <v/>
+      </c>
+      <c r="E38" s="60">
+        <f>D39</f>
+        <v/>
+      </c>
+      <c r="F38" s="60">
+        <f>E39</f>
+        <v/>
+      </c>
+      <c r="G38" s="60">
+        <f>F39</f>
+        <v/>
+      </c>
+      <c r="H38" s="60">
+        <f>G39</f>
+        <v/>
+      </c>
+      <c r="I38" s="60">
+        <f>H39</f>
+        <v/>
+      </c>
+      <c r="J38" s="60">
+        <f>I39</f>
+        <v/>
+      </c>
+      <c r="K38" s="60">
+        <f>J39</f>
+        <v/>
+      </c>
+      <c r="L38" s="60">
+        <f>K39</f>
+        <v/>
+      </c>
+      <c r="M38" s="60">
+        <f>L39</f>
+        <v/>
+      </c>
+      <c r="N38" s="60">
+        <f>M39</f>
+        <v/>
+      </c>
+      <c r="O38" s="60">
+        <f>N39</f>
+        <v/>
+      </c>
+      <c r="P38" s="60">
+        <f>O39</f>
+        <v/>
+      </c>
+      <c r="Q38" s="86">
+        <f>C38</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="51" t="n"/>
-      <c r="B39" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Transfer in from Maybank (top-up to minimum)</t>
-        </is>
-      </c>
-      <c r="C39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-G38)</f>
-        <v/>
-      </c>
-      <c r="H39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-H38)</f>
-        <v/>
-      </c>
-      <c r="I39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-I38)</f>
-        <v/>
-      </c>
-      <c r="J39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-J38)</f>
-        <v/>
-      </c>
-      <c r="K39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-K38)</f>
-        <v/>
-      </c>
-      <c r="L39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-L38)</f>
-        <v/>
-      </c>
-      <c r="M39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-M38)</f>
-        <v/>
-      </c>
-      <c r="N39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-N38)</f>
-        <v/>
-      </c>
-      <c r="O39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-O38)</f>
-        <v/>
-      </c>
-      <c r="P39" s="60">
-        <f>MAX(0,'Q4 Assumptions'!$B$38-P38)</f>
+      <c r="A39" s="80" t="inlineStr">
+        <is>
+          <t>Maybank</t>
+        </is>
+      </c>
+      <c r="B39" s="96" t="inlineStr">
+        <is>
+          <t>Closing balance — Maybank</t>
+        </is>
+      </c>
+      <c r="C39" s="86">
+        <f>C38+C12+C13+C15-SUM(C19:C26)-C36</f>
+        <v/>
+      </c>
+      <c r="D39" s="86">
+        <f>D38+D12+D13+D15-SUM(D19:D26)-D36</f>
+        <v/>
+      </c>
+      <c r="E39" s="86">
+        <f>E38+E12+E13+E15-SUM(E19:E26)-E36</f>
+        <v/>
+      </c>
+      <c r="F39" s="86">
+        <f>F38+F12+F13+F15-SUM(F19:F26)-F36</f>
+        <v/>
+      </c>
+      <c r="G39" s="86">
+        <f>G38+G12+G13+G15-SUM(G19:G26)-G36</f>
+        <v/>
+      </c>
+      <c r="H39" s="86">
+        <f>H38+H12+H13+H15-SUM(H19:H26)-H36</f>
+        <v/>
+      </c>
+      <c r="I39" s="86">
+        <f>I38+I12+I13+I15-SUM(I19:I26)-I36</f>
+        <v/>
+      </c>
+      <c r="J39" s="86">
+        <f>J38+J12+J13+J15-SUM(J19:J26)-J36</f>
+        <v/>
+      </c>
+      <c r="K39" s="86">
+        <f>K38+K12+K13+K15-SUM(K19:K26)-K36</f>
+        <v/>
+      </c>
+      <c r="L39" s="86">
+        <f>L38+L12+L13+L15-SUM(L19:L26)-L36</f>
+        <v/>
+      </c>
+      <c r="M39" s="86">
+        <f>M38+M12+M13+M15-SUM(M19:M26)-M36</f>
+        <v/>
+      </c>
+      <c r="N39" s="86">
+        <f>N38+N12+N13+N15-SUM(N19:N26)-N36</f>
+        <v/>
+      </c>
+      <c r="O39" s="86">
+        <f>O38+O12+O13+O15-SUM(O19:O26)-O36</f>
+        <v/>
+      </c>
+      <c r="P39" s="86">
+        <f>P38+P12+P13+P15-SUM(P19:P26)-P36</f>
         <v/>
       </c>
       <c r="Q39" s="86">
-        <f>SUM(C39:P39)</f>
+        <f>P39</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="51" t="n"/>
-      <c r="B40" s="54" t="inlineStr">
-        <is>
-          <t>Total cash in</t>
-        </is>
-      </c>
-      <c r="C40" s="61">
-        <f>C33+C34+C39</f>
-        <v/>
-      </c>
-      <c r="D40" s="61">
-        <f>D33+D34+D39</f>
-        <v/>
-      </c>
-      <c r="E40" s="61">
-        <f>E33+E34+E39</f>
-        <v/>
-      </c>
-      <c r="F40" s="61">
-        <f>F33+F34+F39</f>
-        <v/>
-      </c>
-      <c r="G40" s="61">
-        <f>G33+G34+G39</f>
-        <v/>
-      </c>
-      <c r="H40" s="61">
-        <f>H33+H34+H39</f>
-        <v/>
-      </c>
-      <c r="I40" s="61">
-        <f>I33+I34+I39</f>
-        <v/>
-      </c>
-      <c r="J40" s="61">
-        <f>J33+J34+J39</f>
-        <v/>
-      </c>
-      <c r="K40" s="61">
-        <f>K33+K34+K39</f>
-        <v/>
-      </c>
-      <c r="L40" s="61">
-        <f>L33+L34+L39</f>
-        <v/>
-      </c>
-      <c r="M40" s="61">
-        <f>M33+M34+M39</f>
-        <v/>
-      </c>
-      <c r="N40" s="61">
-        <f>N33+N34+N39</f>
-        <v/>
-      </c>
-      <c r="O40" s="61">
-        <f>O33+O34+O39</f>
-        <v/>
-      </c>
-      <c r="P40" s="61">
-        <f>P33+P34+P39</f>
-        <v/>
-      </c>
-      <c r="Q40" s="95">
-        <f>SUM(C40:P40)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="51" t="n"/>
-      <c r="B41" s="54" t="inlineStr">
-        <is>
-          <t>Total cash out</t>
-        </is>
-      </c>
-      <c r="C41" s="56">
-        <f>C36+C37</f>
-        <v/>
-      </c>
-      <c r="D41" s="56">
-        <f>D36+D37</f>
-        <v/>
-      </c>
-      <c r="E41" s="56">
-        <f>E36+E37</f>
-        <v/>
-      </c>
-      <c r="F41" s="56">
-        <f>F36+F37</f>
-        <v/>
-      </c>
-      <c r="G41" s="56">
-        <f>G36+G37</f>
-        <v/>
-      </c>
-      <c r="H41" s="56">
-        <f>H36+H37</f>
-        <v/>
-      </c>
-      <c r="I41" s="56">
-        <f>I36+I37</f>
-        <v/>
-      </c>
-      <c r="J41" s="56">
-        <f>J36+J37</f>
-        <v/>
-      </c>
-      <c r="K41" s="56">
-        <f>K36+K37</f>
-        <v/>
-      </c>
-      <c r="L41" s="56">
-        <f>L36+L37</f>
-        <v/>
-      </c>
-      <c r="M41" s="56">
-        <f>M36+M37</f>
-        <v/>
-      </c>
-      <c r="N41" s="56">
-        <f>N36+N37</f>
-        <v/>
-      </c>
-      <c r="O41" s="56">
-        <f>O36+O37</f>
-        <v/>
-      </c>
-      <c r="P41" s="56">
-        <f>P36+P37</f>
-        <v/>
-      </c>
-      <c r="Q41" s="86">
-        <f>SUM(C41:P41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="51" t="n"/>
-      <c r="B42" s="54" t="inlineStr">
-        <is>
-          <t>Net cash flow</t>
-        </is>
-      </c>
-      <c r="C42" s="56">
-        <f>C40-C41</f>
-        <v/>
-      </c>
-      <c r="D42" s="56">
-        <f>D40-D41</f>
-        <v/>
-      </c>
-      <c r="E42" s="56">
-        <f>E40-E41</f>
-        <v/>
-      </c>
-      <c r="F42" s="56">
-        <f>F40-F41</f>
-        <v/>
-      </c>
-      <c r="G42" s="56">
-        <f>G40-G41</f>
-        <v/>
-      </c>
-      <c r="H42" s="56">
-        <f>H40-H41</f>
-        <v/>
-      </c>
-      <c r="I42" s="56">
-        <f>I40-I41</f>
-        <v/>
-      </c>
-      <c r="J42" s="56">
-        <f>J40-J41</f>
-        <v/>
-      </c>
-      <c r="K42" s="56">
-        <f>K40-K41</f>
-        <v/>
-      </c>
-      <c r="L42" s="56">
-        <f>L40-L41</f>
-        <v/>
-      </c>
-      <c r="M42" s="56">
-        <f>M40-M41</f>
-        <v/>
-      </c>
-      <c r="N42" s="56">
-        <f>N40-N41</f>
-        <v/>
-      </c>
-      <c r="O42" s="56">
-        <f>O40-O41</f>
-        <v/>
-      </c>
-      <c r="P42" s="56">
-        <f>P40-P41</f>
-        <v/>
-      </c>
-      <c r="Q42" s="86">
-        <f>SUM(C42:P42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="51" t="n"/>
-      <c r="B43" s="57" t="inlineStr"/>
-      <c r="C43" s="51" t="n"/>
-      <c r="D43" s="51" t="n"/>
-      <c r="E43" s="51" t="n"/>
-      <c r="F43" s="51" t="n"/>
-      <c r="G43" s="51" t="n"/>
-      <c r="H43" s="51" t="n"/>
-      <c r="I43" s="51" t="n"/>
-      <c r="J43" s="51" t="n"/>
-      <c r="K43" s="51" t="n"/>
-      <c r="L43" s="51" t="n"/>
-      <c r="M43" s="51" t="n"/>
-      <c r="N43" s="51" t="n"/>
-      <c r="O43" s="51" t="n"/>
-      <c r="P43" s="51" t="n"/>
-      <c r="Q43" s="51" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="51" t="n"/>
-      <c r="B44" s="96" t="inlineStr">
-        <is>
-          <t>Closing balance — RHB</t>
-        </is>
-      </c>
-      <c r="C44" s="86">
-        <f>C31+C42</f>
-        <v/>
-      </c>
-      <c r="D44" s="86">
-        <f>D31+D42</f>
-        <v/>
-      </c>
-      <c r="E44" s="86">
-        <f>E31+E42</f>
-        <v/>
-      </c>
-      <c r="F44" s="86">
-        <f>F31+F42</f>
-        <v/>
-      </c>
-      <c r="G44" s="86">
-        <f>G31+G42</f>
-        <v/>
-      </c>
-      <c r="H44" s="86">
-        <f>H31+H42</f>
-        <v/>
-      </c>
-      <c r="I44" s="86">
-        <f>I31+I42</f>
-        <v/>
-      </c>
-      <c r="J44" s="86">
-        <f>J31+J42</f>
-        <v/>
-      </c>
-      <c r="K44" s="86">
-        <f>K31+K42</f>
-        <v/>
-      </c>
-      <c r="L44" s="86">
-        <f>L31+L42</f>
-        <v/>
-      </c>
-      <c r="M44" s="86">
-        <f>M31+M42</f>
-        <v/>
-      </c>
-      <c r="N44" s="86">
-        <f>N31+N42</f>
-        <v/>
-      </c>
-      <c r="O44" s="86">
-        <f>O31+O42</f>
-        <v/>
-      </c>
-      <c r="P44" s="86">
-        <f>P31+P42</f>
-        <v/>
-      </c>
-      <c r="Q44" s="86">
-        <f>P44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="51" t="n"/>
-      <c r="B45" s="51" t="n"/>
-      <c r="C45" s="51" t="n"/>
-      <c r="D45" s="51" t="n"/>
-      <c r="E45" s="51" t="n"/>
-      <c r="F45" s="51" t="n"/>
-      <c r="G45" s="51" t="n"/>
-      <c r="H45" s="51" t="n"/>
-      <c r="I45" s="51" t="n"/>
-      <c r="J45" s="51" t="n"/>
-      <c r="K45" s="51" t="n"/>
-      <c r="L45" s="51" t="n"/>
-      <c r="M45" s="51" t="n"/>
-      <c r="N45" s="51" t="n"/>
-      <c r="O45" s="51" t="n"/>
-      <c r="P45" s="51" t="n"/>
-      <c r="Q45" s="51" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="65" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED (MAYBANK + RHB)</t>
-        </is>
-      </c>
-      <c r="B46" s="66" t="n"/>
-      <c r="C46" s="66" t="n"/>
-      <c r="D46" s="66" t="n"/>
-      <c r="E46" s="66" t="n"/>
-      <c r="F46" s="66" t="n"/>
-      <c r="G46" s="66" t="n"/>
-      <c r="H46" s="66" t="n"/>
-      <c r="I46" s="66" t="n"/>
-      <c r="J46" s="66" t="n"/>
-      <c r="K46" s="66" t="n"/>
-      <c r="L46" s="66" t="n"/>
-      <c r="M46" s="66" t="n"/>
-      <c r="N46" s="66" t="n"/>
-      <c r="O46" s="66" t="n"/>
-      <c r="P46" s="66" t="n"/>
-      <c r="Q46" s="66" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="51" t="n"/>
-      <c r="B47" s="54" t="inlineStr">
-        <is>
-          <t>Opening balance</t>
-        </is>
-      </c>
-      <c r="C47" s="56">
-        <f>C10+C31</f>
-        <v/>
-      </c>
-      <c r="D47" s="56">
-        <f>D10+D31</f>
-        <v/>
-      </c>
-      <c r="E47" s="56">
-        <f>E10+E31</f>
-        <v/>
-      </c>
-      <c r="F47" s="56">
-        <f>F10+F31</f>
-        <v/>
-      </c>
-      <c r="G47" s="56">
-        <f>G10+G31</f>
-        <v/>
-      </c>
-      <c r="H47" s="56">
-        <f>H10+H31</f>
-        <v/>
-      </c>
-      <c r="I47" s="56">
-        <f>I10+I31</f>
-        <v/>
-      </c>
-      <c r="J47" s="56">
-        <f>J10+J31</f>
-        <v/>
-      </c>
-      <c r="K47" s="56">
-        <f>K10+K31</f>
-        <v/>
-      </c>
-      <c r="L47" s="56">
-        <f>L10+L31</f>
-        <v/>
-      </c>
-      <c r="M47" s="56">
-        <f>M10+M31</f>
-        <v/>
-      </c>
-      <c r="N47" s="56">
-        <f>N10+N31</f>
-        <v/>
-      </c>
-      <c r="O47" s="56">
-        <f>O10+O31</f>
-        <v/>
-      </c>
-      <c r="P47" s="56">
-        <f>P10+P31</f>
-        <v/>
-      </c>
-      <c r="Q47" s="86">
-        <f>C47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="51" t="n"/>
-      <c r="B48" s="54" t="inlineStr">
-        <is>
-          <t>Net cash flow (excl. inter-bank transfers)</t>
-        </is>
-      </c>
-      <c r="C48" s="56">
-        <f>C27+C42</f>
-        <v/>
-      </c>
-      <c r="D48" s="56">
-        <f>D27+D42</f>
-        <v/>
-      </c>
-      <c r="E48" s="56">
-        <f>E27+E42</f>
-        <v/>
-      </c>
-      <c r="F48" s="56">
-        <f>F27+F42</f>
-        <v/>
-      </c>
-      <c r="G48" s="56">
-        <f>G27+G42</f>
-        <v/>
-      </c>
-      <c r="H48" s="56">
-        <f>H27+H42</f>
-        <v/>
-      </c>
-      <c r="I48" s="56">
-        <f>I27+I42</f>
-        <v/>
-      </c>
-      <c r="J48" s="56">
-        <f>J27+J42</f>
-        <v/>
-      </c>
-      <c r="K48" s="56">
-        <f>K27+K42</f>
-        <v/>
-      </c>
-      <c r="L48" s="56">
-        <f>L27+L42</f>
-        <v/>
-      </c>
-      <c r="M48" s="56">
-        <f>M27+M42</f>
-        <v/>
-      </c>
-      <c r="N48" s="56">
-        <f>N27+N42</f>
-        <v/>
-      </c>
-      <c r="O48" s="56">
-        <f>O27+O42</f>
-        <v/>
-      </c>
-      <c r="P48" s="56">
-        <f>P27+P42</f>
-        <v/>
-      </c>
-      <c r="Q48" s="86">
-        <f>SUM(C48:P48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="51" t="n"/>
-      <c r="B49" s="96" t="inlineStr">
-        <is>
-          <t>Closing balance — combined</t>
-        </is>
-      </c>
-      <c r="C49" s="86">
-        <f>C28+C44</f>
-        <v/>
-      </c>
-      <c r="D49" s="86">
-        <f>D28+D44</f>
-        <v/>
-      </c>
-      <c r="E49" s="86">
-        <f>E28+E44</f>
-        <v/>
-      </c>
-      <c r="F49" s="86">
-        <f>F28+F44</f>
-        <v/>
-      </c>
-      <c r="G49" s="86">
-        <f>G28+G44</f>
-        <v/>
-      </c>
-      <c r="H49" s="86">
-        <f>H28+H44</f>
-        <v/>
-      </c>
-      <c r="I49" s="86">
-        <f>I28+I44</f>
-        <v/>
-      </c>
-      <c r="J49" s="86">
-        <f>J28+J44</f>
-        <v/>
-      </c>
-      <c r="K49" s="86">
-        <f>K28+K44</f>
-        <v/>
-      </c>
-      <c r="L49" s="86">
-        <f>L28+L44</f>
-        <v/>
-      </c>
-      <c r="M49" s="86">
-        <f>M28+M44</f>
-        <v/>
-      </c>
-      <c r="N49" s="86">
-        <f>N28+N44</f>
-        <v/>
-      </c>
-      <c r="O49" s="86">
-        <f>O28+O44</f>
-        <v/>
-      </c>
-      <c r="P49" s="86">
-        <f>P28+P44</f>
-        <v/>
-      </c>
-      <c r="Q49" s="86">
-        <f>P49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="51" t="n"/>
-      <c r="B50" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Check: opening + net − closing (should be 0)</t>
-        </is>
-      </c>
-      <c r="C50" s="64">
-        <f>ROUND(C47+C48-C49,2)</f>
-        <v/>
-      </c>
-      <c r="D50" s="64">
-        <f>ROUND(D47+D48-D49,2)</f>
-        <v/>
-      </c>
-      <c r="E50" s="64">
-        <f>ROUND(E47+E48-E49,2)</f>
-        <v/>
-      </c>
-      <c r="F50" s="64">
-        <f>ROUND(F47+F48-F49,2)</f>
-        <v/>
-      </c>
-      <c r="G50" s="64">
-        <f>ROUND(G47+G48-G49,2)</f>
-        <v/>
-      </c>
-      <c r="H50" s="64">
-        <f>ROUND(H47+H48-H49,2)</f>
-        <v/>
-      </c>
-      <c r="I50" s="64">
-        <f>ROUND(I47+I48-I49,2)</f>
-        <v/>
-      </c>
-      <c r="J50" s="64">
-        <f>ROUND(J47+J48-J49,2)</f>
-        <v/>
-      </c>
-      <c r="K50" s="64">
-        <f>ROUND(K47+K48-K49,2)</f>
-        <v/>
-      </c>
-      <c r="L50" s="64">
-        <f>ROUND(L47+L48-L49,2)</f>
-        <v/>
-      </c>
-      <c r="M50" s="64">
-        <f>ROUND(M47+M48-M49,2)</f>
-        <v/>
-      </c>
-      <c r="N50" s="64">
-        <f>ROUND(N47+N48-N49,2)</f>
-        <v/>
-      </c>
-      <c r="O50" s="64">
-        <f>ROUND(O47+O48-O49,2)</f>
-        <v/>
-      </c>
-      <c r="P50" s="64">
-        <f>ROUND(P47+P48-P49,2)</f>
-        <v/>
-      </c>
-      <c r="Q50" s="51" t="n"/>
+      <c r="B40" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Check: Maybank + RHB − combined closing (should be 0)</t>
+        </is>
+      </c>
+      <c r="C40" s="64">
+        <f>ROUND(C37+C39-C31,2)</f>
+        <v/>
+      </c>
+      <c r="D40" s="64">
+        <f>ROUND(D37+D39-D31,2)</f>
+        <v/>
+      </c>
+      <c r="E40" s="64">
+        <f>ROUND(E37+E39-E31,2)</f>
+        <v/>
+      </c>
+      <c r="F40" s="64">
+        <f>ROUND(F37+F39-F31,2)</f>
+        <v/>
+      </c>
+      <c r="G40" s="64">
+        <f>ROUND(G37+G39-G31,2)</f>
+        <v/>
+      </c>
+      <c r="H40" s="64">
+        <f>ROUND(H37+H39-H31,2)</f>
+        <v/>
+      </c>
+      <c r="I40" s="64">
+        <f>ROUND(I37+I39-I31,2)</f>
+        <v/>
+      </c>
+      <c r="J40" s="64">
+        <f>ROUND(J37+J39-J31,2)</f>
+        <v/>
+      </c>
+      <c r="K40" s="64">
+        <f>ROUND(K37+K39-K31,2)</f>
+        <v/>
+      </c>
+      <c r="L40" s="64">
+        <f>ROUND(L37+L39-L31,2)</f>
+        <v/>
+      </c>
+      <c r="M40" s="64">
+        <f>ROUND(M37+M39-M31,2)</f>
+        <v/>
+      </c>
+      <c r="N40" s="64">
+        <f>ROUND(N37+N39-N31,2)</f>
+        <v/>
+      </c>
+      <c r="O40" s="64">
+        <f>ROUND(O37+O39-O31,2)</f>
+        <v/>
+      </c>
+      <c r="P40" s="64">
+        <f>ROUND(P37+P39-P31,2)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="51" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add utilities increase of 3% per new outlet to Q4 forecast
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141mGWEWvuV7DFAd6Wzc4uL
</commit_message>
<xml_diff>
--- a/TGFB_Q4_2026_Weekly_CashFlow_Forecast.xlsx
+++ b/TGFB_Q4_2026_Weekly_CashFlow_Forecast.xlsx
@@ -549,7 +549,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Q4 Weekly Cash Flow'!$D$99:$Q$99</f>
+              <f>'Q4 Weekly Cash Flow'!$D$100:$Q$100</f>
             </numRef>
           </val>
         </ser>
@@ -596,7 +596,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>102</row>
+      <row>103</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="2880000"/>
@@ -896,7 +896,7 @@
         <v/>
       </c>
       <c r="C7" s="58">
-        <f>'Q4 Weekly Cash Flow'!R94+'Q4 Weekly Cash Flow'!R95</f>
+        <f>'Q4 Weekly Cash Flow'!R95+'Q4 Weekly Cash Flow'!R96</f>
         <v/>
       </c>
       <c r="D7" s="58">
@@ -947,11 +947,11 @@
         </is>
       </c>
       <c r="B10" s="58">
-        <f>-'Q4 Weekly Cash Flow'!R97</f>
+        <f>-'Q4 Weekly Cash Flow'!R98</f>
         <v/>
       </c>
       <c r="C10" s="58">
-        <f>'Q4 Weekly Cash Flow'!R97</f>
+        <f>'Q4 Weekly Cash Flow'!R98</f>
         <v/>
       </c>
       <c r="D10" s="57">
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="B13" s="63">
-        <f>ROUND(B12-'Q4 Weekly Cash Flow'!R99,2)</f>
+        <f>ROUND(B12-'Q4 Weekly Cash Flow'!R100,2)</f>
         <v/>
       </c>
       <c r="C13" s="63">
-        <f>ROUND(C12-'Q4 Weekly Cash Flow'!R98,2)</f>
+        <f>ROUND(C12-'Q4 Weekly Cash Flow'!R99,2)</f>
         <v/>
       </c>
       <c r="D13" s="63">
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="B18" s="57">
-        <f>MIN('Q4 Weekly Cash Flow'!$D$99:$Q$99)</f>
+        <f>MIN('Q4 Weekly Cash Flow'!$D$100:$Q$100)</f>
         <v/>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="D21" s="57">
-        <f>-'Q4 Weekly Cash Flow'!R89</f>
+        <f>-'Q4 Weekly Cash Flow'!R90</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="68" t="inlineStr">
         <is>
-          <t>4. New outlets: RM8k/day sales; each new outlet open adds +3% to inventory purchases and +1% to branch upkeep (on the Sep daily level); rental 5% of new-outlet sales. Bebeks RM400k mid-Oct, Kopitiam RM350k on 31 Dec.</t>
+          <t>4. New outlets: RM8k/day sales; each new outlet open adds +3% to inventory purchases and +1% to branch upkeep and +3% to utilities (on the Sep daily level); rental 5% of new-outlet sales. Bebeks RM400k mid-Oct, Kopitiam RM350k on 31 Dec.</t>
         </is>
       </c>
       <c r="B27" s="1" t="n"/>
@@ -5480,6 +5480,21 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="56" t="inlineStr">
+        <is>
+          <t>Utilities increase per new outlet open</t>
+        </is>
+      </c>
+      <c r="B25" s="82" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I25" s="52" t="inlineStr">
+        <is>
+          <t>Your instruction: +3% per new outlet</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" s="64" t="inlineStr">
         <is>
@@ -8710,7 +8725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R101"/>
+  <dimension ref="A1:R102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9125,59 +9140,59 @@
         <v/>
       </c>
       <c r="D14" s="103">
-        <f>'Q4 Assumptions'!$G$36*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D83+D90</f>
+        <f>'Q4 Assumptions'!$G$36*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D83+D91</f>
         <v/>
       </c>
       <c r="E14" s="103">
-        <f>'Q4 Assumptions'!$G$36*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E83+E90</f>
+        <f>'Q4 Assumptions'!$G$36*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E83+E91</f>
         <v/>
       </c>
       <c r="F14" s="103">
-        <f>'Q4 Assumptions'!$G$36*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F83+F90</f>
+        <f>'Q4 Assumptions'!$G$36*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F83+F91</f>
         <v/>
       </c>
       <c r="G14" s="103">
-        <f>'Q4 Assumptions'!$G$36*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G83+G90</f>
+        <f>'Q4 Assumptions'!$G$36*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G83+G91</f>
         <v/>
       </c>
       <c r="H14" s="103">
-        <f>'Q4 Assumptions'!$G$36*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H83+H90</f>
+        <f>'Q4 Assumptions'!$G$36*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H83+H91</f>
         <v/>
       </c>
       <c r="I14" s="103">
-        <f>'Q4 Assumptions'!$G$36*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I83+I90</f>
+        <f>'Q4 Assumptions'!$G$36*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I83+I91</f>
         <v/>
       </c>
       <c r="J14" s="103">
-        <f>'Q4 Assumptions'!$G$36*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J83+J90</f>
+        <f>'Q4 Assumptions'!$G$36*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J83+J91</f>
         <v/>
       </c>
       <c r="K14" s="103">
-        <f>'Q4 Assumptions'!$G$36*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K83+K90</f>
+        <f>'Q4 Assumptions'!$G$36*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K83+K91</f>
         <v/>
       </c>
       <c r="L14" s="103">
-        <f>'Q4 Assumptions'!$G$36*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L83+L90</f>
+        <f>'Q4 Assumptions'!$G$36*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L83+L91</f>
         <v/>
       </c>
       <c r="M14" s="103">
-        <f>'Q4 Assumptions'!$G$36*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M83+M90</f>
+        <f>'Q4 Assumptions'!$G$36*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M83+M91</f>
         <v/>
       </c>
       <c r="N14" s="103">
-        <f>'Q4 Assumptions'!$G$36*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N83+N90</f>
+        <f>'Q4 Assumptions'!$G$36*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N83+N91</f>
         <v/>
       </c>
       <c r="O14" s="103">
-        <f>'Q4 Assumptions'!$G$36*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O83+O90</f>
+        <f>'Q4 Assumptions'!$G$36*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O83+O91</f>
         <v/>
       </c>
       <c r="P14" s="103">
-        <f>'Q4 Assumptions'!$G$36*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P83+P90</f>
+        <f>'Q4 Assumptions'!$G$36*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P83+P91</f>
         <v/>
       </c>
       <c r="Q14" s="103">
-        <f>'Q4 Assumptions'!$G$36*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q83+Q90</f>
+        <f>'Q4 Assumptions'!$G$36*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$36,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q83+Q91</f>
         <v/>
       </c>
       <c r="R14" s="104">
@@ -10657,59 +10672,59 @@
         <v/>
       </c>
       <c r="D36" s="103">
-        <f>'Q4 Assumptions'!$G$56*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)</f>
+        <f>'Q4 Assumptions'!$G$56*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D88</f>
         <v/>
       </c>
       <c r="E36" s="103">
-        <f>'Q4 Assumptions'!$G$56*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)</f>
+        <f>'Q4 Assumptions'!$G$56*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E88</f>
         <v/>
       </c>
       <c r="F36" s="103">
-        <f>'Q4 Assumptions'!$G$56*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)</f>
+        <f>'Q4 Assumptions'!$G$56*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F88</f>
         <v/>
       </c>
       <c r="G36" s="103">
-        <f>'Q4 Assumptions'!$G$56*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)</f>
+        <f>'Q4 Assumptions'!$G$56*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G88</f>
         <v/>
       </c>
       <c r="H36" s="103">
-        <f>'Q4 Assumptions'!$G$56*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)</f>
+        <f>'Q4 Assumptions'!$G$56*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H88</f>
         <v/>
       </c>
       <c r="I36" s="103">
-        <f>'Q4 Assumptions'!$G$56*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)</f>
+        <f>'Q4 Assumptions'!$G$56*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I88</f>
         <v/>
       </c>
       <c r="J36" s="103">
-        <f>'Q4 Assumptions'!$G$56*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)</f>
+        <f>'Q4 Assumptions'!$G$56*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J88</f>
         <v/>
       </c>
       <c r="K36" s="103">
-        <f>'Q4 Assumptions'!$G$56*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)</f>
+        <f>'Q4 Assumptions'!$G$56*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K88</f>
         <v/>
       </c>
       <c r="L36" s="103">
-        <f>'Q4 Assumptions'!$G$56*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)</f>
+        <f>'Q4 Assumptions'!$G$56*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L88</f>
         <v/>
       </c>
       <c r="M36" s="103">
-        <f>'Q4 Assumptions'!$G$56*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)</f>
+        <f>'Q4 Assumptions'!$G$56*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M88</f>
         <v/>
       </c>
       <c r="N36" s="103">
-        <f>'Q4 Assumptions'!$G$56*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)</f>
+        <f>'Q4 Assumptions'!$G$56*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N88</f>
         <v/>
       </c>
       <c r="O36" s="103">
-        <f>'Q4 Assumptions'!$G$56*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)</f>
+        <f>'Q4 Assumptions'!$G$56*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O88</f>
         <v/>
       </c>
       <c r="P36" s="103">
-        <f>'Q4 Assumptions'!$G$56*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)</f>
+        <f>'Q4 Assumptions'!$G$56*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P88</f>
         <v/>
       </c>
       <c r="Q36" s="103">
-        <f>'Q4 Assumptions'!$G$56*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)</f>
+        <f>'Q4 Assumptions'!$G$56*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$56,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q88</f>
         <v/>
       </c>
       <c r="R36" s="104">
@@ -10729,59 +10744,59 @@
         <v/>
       </c>
       <c r="D37" s="103">
-        <f>'Q4 Assumptions'!$G$57*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D88</f>
+        <f>'Q4 Assumptions'!$G$57*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D89</f>
         <v/>
       </c>
       <c r="E37" s="103">
-        <f>'Q4 Assumptions'!$G$57*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E88</f>
+        <f>'Q4 Assumptions'!$G$57*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E89</f>
         <v/>
       </c>
       <c r="F37" s="103">
-        <f>'Q4 Assumptions'!$G$57*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F88</f>
+        <f>'Q4 Assumptions'!$G$57*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F89</f>
         <v/>
       </c>
       <c r="G37" s="103">
-        <f>'Q4 Assumptions'!$G$57*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G88</f>
+        <f>'Q4 Assumptions'!$G$57*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G89</f>
         <v/>
       </c>
       <c r="H37" s="103">
-        <f>'Q4 Assumptions'!$G$57*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H88</f>
+        <f>'Q4 Assumptions'!$G$57*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H89</f>
         <v/>
       </c>
       <c r="I37" s="103">
-        <f>'Q4 Assumptions'!$G$57*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I88</f>
+        <f>'Q4 Assumptions'!$G$57*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I89</f>
         <v/>
       </c>
       <c r="J37" s="103">
-        <f>'Q4 Assumptions'!$G$57*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J88</f>
+        <f>'Q4 Assumptions'!$G$57*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J89</f>
         <v/>
       </c>
       <c r="K37" s="103">
-        <f>'Q4 Assumptions'!$G$57*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K88</f>
+        <f>'Q4 Assumptions'!$G$57*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K89</f>
         <v/>
       </c>
       <c r="L37" s="103">
-        <f>'Q4 Assumptions'!$G$57*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L88</f>
+        <f>'Q4 Assumptions'!$G$57*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L89</f>
         <v/>
       </c>
       <c r="M37" s="103">
-        <f>'Q4 Assumptions'!$G$57*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M88</f>
+        <f>'Q4 Assumptions'!$G$57*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M89</f>
         <v/>
       </c>
       <c r="N37" s="103">
-        <f>'Q4 Assumptions'!$G$57*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N88</f>
+        <f>'Q4 Assumptions'!$G$57*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N89</f>
         <v/>
       </c>
       <c r="O37" s="103">
-        <f>'Q4 Assumptions'!$G$57*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O88</f>
+        <f>'Q4 Assumptions'!$G$57*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O89</f>
         <v/>
       </c>
       <c r="P37" s="103">
-        <f>'Q4 Assumptions'!$G$57*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P88</f>
+        <f>'Q4 Assumptions'!$G$57*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P89</f>
         <v/>
       </c>
       <c r="Q37" s="103">
-        <f>'Q4 Assumptions'!$G$57*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q88</f>
+        <f>'Q4 Assumptions'!$G$57*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$57,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q89</f>
         <v/>
       </c>
       <c r="R37" s="104">
@@ -11593,59 +11608,59 @@
         <v/>
       </c>
       <c r="D53" s="103">
-        <f>'Q4 Assumptions'!$G$67*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D89</f>
+        <f>'Q4 Assumptions'!$G$67*D$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+D90</f>
         <v/>
       </c>
       <c r="E53" s="103">
-        <f>'Q4 Assumptions'!$G$67*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E89</f>
+        <f>'Q4 Assumptions'!$G$67*E$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+E90</f>
         <v/>
       </c>
       <c r="F53" s="103">
-        <f>'Q4 Assumptions'!$G$67*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F89</f>
+        <f>'Q4 Assumptions'!$G$67*F$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+F90</f>
         <v/>
       </c>
       <c r="G53" s="103">
-        <f>'Q4 Assumptions'!$G$67*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G89</f>
+        <f>'Q4 Assumptions'!$G$67*G$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+G90</f>
         <v/>
       </c>
       <c r="H53" s="103">
-        <f>'Q4 Assumptions'!$G$67*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H89</f>
+        <f>'Q4 Assumptions'!$G$67*H$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+H90</f>
         <v/>
       </c>
       <c r="I53" s="103">
-        <f>'Q4 Assumptions'!$G$67*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I89</f>
+        <f>'Q4 Assumptions'!$G$67*I$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+I90</f>
         <v/>
       </c>
       <c r="J53" s="103">
-        <f>'Q4 Assumptions'!$G$67*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J89</f>
+        <f>'Q4 Assumptions'!$G$67*J$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+J90</f>
         <v/>
       </c>
       <c r="K53" s="103">
-        <f>'Q4 Assumptions'!$G$67*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K89</f>
+        <f>'Q4 Assumptions'!$G$67*K$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+K90</f>
         <v/>
       </c>
       <c r="L53" s="103">
-        <f>'Q4 Assumptions'!$G$67*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L89</f>
+        <f>'Q4 Assumptions'!$G$67*L$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+L90</f>
         <v/>
       </c>
       <c r="M53" s="103">
-        <f>'Q4 Assumptions'!$G$67*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M89</f>
+        <f>'Q4 Assumptions'!$G$67*M$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+M90</f>
         <v/>
       </c>
       <c r="N53" s="103">
-        <f>'Q4 Assumptions'!$G$67*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N89</f>
+        <f>'Q4 Assumptions'!$G$67*N$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+N90</f>
         <v/>
       </c>
       <c r="O53" s="103">
-        <f>'Q4 Assumptions'!$G$67*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O89</f>
+        <f>'Q4 Assumptions'!$G$67*O$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+O90</f>
         <v/>
       </c>
       <c r="P53" s="103">
-        <f>'Q4 Assumptions'!$G$67*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P89</f>
+        <f>'Q4 Assumptions'!$G$67*P$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+P90</f>
         <v/>
       </c>
       <c r="Q53" s="103">
-        <f>'Q4 Assumptions'!$G$67*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q89</f>
+        <f>'Q4 Assumptions'!$G$67*Q$12+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$D$85:$D$133,'Q4 Assumptions'!$A$67,'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+Q90</f>
         <v/>
       </c>
       <c r="R53" s="104">
@@ -13032,63 +13047,63 @@
         <v/>
       </c>
       <c r="D78" s="85">
-        <f>D99</f>
+        <f>D100</f>
         <v/>
       </c>
       <c r="E78" s="85">
-        <f>E99</f>
+        <f>E100</f>
         <v/>
       </c>
       <c r="F78" s="85">
-        <f>F99</f>
+        <f>F100</f>
         <v/>
       </c>
       <c r="G78" s="85">
-        <f>G99</f>
+        <f>G100</f>
         <v/>
       </c>
       <c r="H78" s="85">
-        <f>H99</f>
+        <f>H100</f>
         <v/>
       </c>
       <c r="I78" s="85">
-        <f>I99</f>
+        <f>I100</f>
         <v/>
       </c>
       <c r="J78" s="85">
-        <f>J99</f>
+        <f>J100</f>
         <v/>
       </c>
       <c r="K78" s="85">
-        <f>K99</f>
+        <f>K100</f>
         <v/>
       </c>
       <c r="L78" s="85">
-        <f>L99</f>
+        <f>L100</f>
         <v/>
       </c>
       <c r="M78" s="85">
-        <f>M99</f>
+        <f>M100</f>
         <v/>
       </c>
       <c r="N78" s="85">
-        <f>N99</f>
+        <f>N100</f>
         <v/>
       </c>
       <c r="O78" s="85">
-        <f>O99</f>
+        <f>O100</f>
         <v/>
       </c>
       <c r="P78" s="85">
-        <f>P99</f>
+        <f>P100</f>
         <v/>
       </c>
       <c r="Q78" s="85">
-        <f>Q99</f>
+        <f>Q100</f>
         <v/>
       </c>
       <c r="R78" s="85">
-        <f>R99</f>
+        <f>R100</f>
         <v/>
       </c>
     </row>
@@ -13104,63 +13119,63 @@
         </is>
       </c>
       <c r="D79" s="85">
-        <f>D98</f>
+        <f>D99</f>
         <v/>
       </c>
       <c r="E79" s="85">
-        <f>E98</f>
+        <f>E99</f>
         <v/>
       </c>
       <c r="F79" s="85">
-        <f>F98</f>
+        <f>F99</f>
         <v/>
       </c>
       <c r="G79" s="85">
-        <f>G98</f>
+        <f>G99</f>
         <v/>
       </c>
       <c r="H79" s="85">
-        <f>H98</f>
+        <f>H99</f>
         <v/>
       </c>
       <c r="I79" s="85">
-        <f>I98</f>
+        <f>I99</f>
         <v/>
       </c>
       <c r="J79" s="85">
-        <f>J98</f>
+        <f>J99</f>
         <v/>
       </c>
       <c r="K79" s="85">
-        <f>K98</f>
+        <f>K99</f>
         <v/>
       </c>
       <c r="L79" s="85">
-        <f>L98</f>
+        <f>L99</f>
         <v/>
       </c>
       <c r="M79" s="85">
-        <f>M98</f>
+        <f>M99</f>
         <v/>
       </c>
       <c r="N79" s="85">
-        <f>N98</f>
+        <f>N99</f>
         <v/>
       </c>
       <c r="O79" s="85">
-        <f>O98</f>
+        <f>O99</f>
         <v/>
       </c>
       <c r="P79" s="85">
-        <f>P98</f>
+        <f>P99</f>
         <v/>
       </c>
       <c r="Q79" s="85">
-        <f>Q98</f>
+        <f>Q99</f>
         <v/>
       </c>
       <c r="R79" s="85">
-        <f>R98</f>
+        <f>R99</f>
         <v/>
       </c>
     </row>
@@ -13522,63 +13537,63 @@
     <row r="88">
       <c r="A88" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   New-outlet rental 5% of sales (in Rental)</t>
+          <t xml:space="preserve">   Utilities increase +3% per new outlet (in Utilities)</t>
         </is>
       </c>
       <c r="D88" s="85">
-        <f>-D83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*D$12*'Q4 Assumptions'!$B$25*D84</f>
         <v/>
       </c>
       <c r="E88" s="85">
-        <f>-E83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*E$12*'Q4 Assumptions'!$B$25*E84</f>
         <v/>
       </c>
       <c r="F88" s="85">
-        <f>-F83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*F$12*'Q4 Assumptions'!$B$25*F84</f>
         <v/>
       </c>
       <c r="G88" s="85">
-        <f>-G83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*G$12*'Q4 Assumptions'!$B$25*G84</f>
         <v/>
       </c>
       <c r="H88" s="85">
-        <f>-H83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*H$12*'Q4 Assumptions'!$B$25*H84</f>
         <v/>
       </c>
       <c r="I88" s="85">
-        <f>-I83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*I$12*'Q4 Assumptions'!$B$25*I84</f>
         <v/>
       </c>
       <c r="J88" s="85">
-        <f>-J83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*J$12*'Q4 Assumptions'!$B$25*J84</f>
         <v/>
       </c>
       <c r="K88" s="85">
-        <f>-K83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*K$12*'Q4 Assumptions'!$B$25*K84</f>
         <v/>
       </c>
       <c r="L88" s="85">
-        <f>-L83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*L$12*'Q4 Assumptions'!$B$25*L84</f>
         <v/>
       </c>
       <c r="M88" s="85">
-        <f>-M83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*M$12*'Q4 Assumptions'!$B$25*M84</f>
         <v/>
       </c>
       <c r="N88" s="85">
-        <f>-N83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*N$12*'Q4 Assumptions'!$B$25*N84</f>
         <v/>
       </c>
       <c r="O88" s="85">
-        <f>-O83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*O$12*'Q4 Assumptions'!$B$25*O84</f>
         <v/>
       </c>
       <c r="P88" s="85">
-        <f>-P83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*P$12*'Q4 Assumptions'!$B$25*P84</f>
         <v/>
       </c>
       <c r="Q88" s="85">
-        <f>-Q83*'Q4 Assumptions'!$B$14</f>
+        <f>'Q4 Assumptions'!$G$56*Q$12*'Q4 Assumptions'!$B$25*Q84</f>
         <v/>
       </c>
       <c r="R88" s="93">
@@ -13589,63 +13604,63 @@
     <row r="89">
       <c r="A89" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Capex new outlets (Capex New Branches)</t>
+          <t xml:space="preserve">   New-outlet rental 5% of sales (in Rental)</t>
         </is>
       </c>
       <c r="D89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;D$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;D$11)</f>
+        <f>-D83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="E89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;E$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;E$11)</f>
+        <f>-E83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="F89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;F$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;F$11)</f>
+        <f>-F83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="G89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;G$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;G$11)</f>
+        <f>-G83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="H89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;H$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;H$11)</f>
+        <f>-H83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="I89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;I$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;I$11)</f>
+        <f>-I83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="J89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;J$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;J$11)</f>
+        <f>-J83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="K89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;K$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;K$11)</f>
+        <f>-K83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="L89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;L$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;L$11)</f>
+        <f>-L83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="M89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;M$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;M$11)</f>
+        <f>-M83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="N89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;N$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;N$11)</f>
+        <f>-N83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="O89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;O$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;O$11)</f>
+        <f>-O83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="P89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;P$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;P$11)</f>
+        <f>-P83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="Q89" s="85">
-        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;Q$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;Q$11)</f>
+        <f>-Q83*'Q4 Assumptions'!$B$14</f>
         <v/>
       </c>
       <c r="R89" s="93">
@@ -13656,63 +13671,63 @@
     <row r="90">
       <c r="A90" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   RHB cash deposits (in Customers &amp; Sales)</t>
+          <t xml:space="preserve">   Capex new outlets (Capex New Branches)</t>
         </is>
       </c>
       <c r="D90" s="85">
-        <f>'Q4 Assumptions'!$B$27*D$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;D$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;D$11)</f>
         <v/>
       </c>
       <c r="E90" s="85">
-        <f>'Q4 Assumptions'!$B$27*E$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;E$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;E$11)</f>
         <v/>
       </c>
       <c r="F90" s="85">
-        <f>'Q4 Assumptions'!$B$27*F$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;F$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;F$11)</f>
         <v/>
       </c>
       <c r="G90" s="85">
-        <f>'Q4 Assumptions'!$B$27*G$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;G$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;G$11)</f>
         <v/>
       </c>
       <c r="H90" s="85">
-        <f>'Q4 Assumptions'!$B$27*H$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;H$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;H$11)</f>
         <v/>
       </c>
       <c r="I90" s="85">
-        <f>'Q4 Assumptions'!$B$27*I$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;I$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;I$11)</f>
         <v/>
       </c>
       <c r="J90" s="85">
-        <f>'Q4 Assumptions'!$B$27*J$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;J$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;J$11)</f>
         <v/>
       </c>
       <c r="K90" s="85">
-        <f>'Q4 Assumptions'!$B$27*K$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;K$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;K$11)</f>
         <v/>
       </c>
       <c r="L90" s="85">
-        <f>'Q4 Assumptions'!$B$27*L$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;L$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;L$11)</f>
         <v/>
       </c>
       <c r="M90" s="85">
-        <f>'Q4 Assumptions'!$B$27*M$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;M$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;M$11)</f>
         <v/>
       </c>
       <c r="N90" s="85">
-        <f>'Q4 Assumptions'!$B$27*N$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;N$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;N$11)</f>
         <v/>
       </c>
       <c r="O90" s="85">
-        <f>'Q4 Assumptions'!$B$27*O$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;O$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;O$11)</f>
         <v/>
       </c>
       <c r="P90" s="85">
-        <f>'Q4 Assumptions'!$B$27*P$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;P$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;P$11)</f>
         <v/>
       </c>
       <c r="Q90" s="85">
-        <f>'Q4 Assumptions'!$B$27*Q$12</f>
+        <f>-SUMIFS('Q4 Outlet Schedule'!$F$6:$F$17,'Q4 Outlet Schedule'!$G$6:$G$17,"&gt;="&amp;Q$10,'Q4 Outlet Schedule'!$G$6:$G$17,"&lt;="&amp;Q$11)</f>
         <v/>
       </c>
       <c r="R90" s="93">
@@ -13720,224 +13735,224 @@
         <v/>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="64" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   RHB cash deposits (in Customers &amp; Sales)</t>
+        </is>
+      </c>
+      <c r="D91" s="85">
+        <f>'Q4 Assumptions'!$B$27*D$12</f>
+        <v/>
+      </c>
+      <c r="E91" s="85">
+        <f>'Q4 Assumptions'!$B$27*E$12</f>
+        <v/>
+      </c>
+      <c r="F91" s="85">
+        <f>'Q4 Assumptions'!$B$27*F$12</f>
+        <v/>
+      </c>
+      <c r="G91" s="85">
+        <f>'Q4 Assumptions'!$B$27*G$12</f>
+        <v/>
+      </c>
+      <c r="H91" s="85">
+        <f>'Q4 Assumptions'!$B$27*H$12</f>
+        <v/>
+      </c>
+      <c r="I91" s="85">
+        <f>'Q4 Assumptions'!$B$27*I$12</f>
+        <v/>
+      </c>
+      <c r="J91" s="85">
+        <f>'Q4 Assumptions'!$B$27*J$12</f>
+        <v/>
+      </c>
+      <c r="K91" s="85">
+        <f>'Q4 Assumptions'!$B$27*K$12</f>
+        <v/>
+      </c>
+      <c r="L91" s="85">
+        <f>'Q4 Assumptions'!$B$27*L$12</f>
+        <v/>
+      </c>
+      <c r="M91" s="85">
+        <f>'Q4 Assumptions'!$B$27*M$12</f>
+        <v/>
+      </c>
+      <c r="N91" s="85">
+        <f>'Q4 Assumptions'!$B$27*N$12</f>
+        <v/>
+      </c>
+      <c r="O91" s="85">
+        <f>'Q4 Assumptions'!$B$27*O$12</f>
+        <v/>
+      </c>
+      <c r="P91" s="85">
+        <f>'Q4 Assumptions'!$B$27*P$12</f>
+        <v/>
+      </c>
+      <c r="Q91" s="85">
+        <f>'Q4 Assumptions'!$B$27*Q$12</f>
+        <v/>
+      </c>
+      <c r="R91" s="93">
+        <f>SUM(D91:Q91)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="64" t="inlineStr">
         <is>
           <t>SPLIT BY BANK — RHB is topped up from Maybank only when payroll needs it (transfer nets to zero combined)</t>
         </is>
       </c>
-      <c r="B92" s="65" t="n"/>
-      <c r="C92" s="65" t="n"/>
-      <c r="D92" s="65" t="n"/>
-      <c r="E92" s="65" t="n"/>
-      <c r="F92" s="65" t="n"/>
-      <c r="G92" s="65" t="n"/>
-      <c r="H92" s="65" t="n"/>
-      <c r="I92" s="65" t="n"/>
-      <c r="J92" s="65" t="n"/>
-      <c r="K92" s="65" t="n"/>
-      <c r="L92" s="65" t="n"/>
-      <c r="M92" s="65" t="n"/>
-      <c r="N92" s="65" t="n"/>
-      <c r="O92" s="65" t="n"/>
-      <c r="P92" s="65" t="n"/>
-      <c r="Q92" s="65" t="n"/>
-      <c r="R92" s="65" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   RHB opening balance</t>
-        </is>
-      </c>
-      <c r="D93" s="85">
-        <f>'Q4 Assumptions'!$B$8</f>
-        <v/>
-      </c>
-      <c r="E93" s="85">
-        <f>D98</f>
-        <v/>
-      </c>
-      <c r="F93" s="85">
-        <f>E98</f>
-        <v/>
-      </c>
-      <c r="G93" s="85">
-        <f>F98</f>
-        <v/>
-      </c>
-      <c r="H93" s="85">
-        <f>G98</f>
-        <v/>
-      </c>
-      <c r="I93" s="85">
-        <f>H98</f>
-        <v/>
-      </c>
-      <c r="J93" s="85">
-        <f>I98</f>
-        <v/>
-      </c>
-      <c r="K93" s="85">
-        <f>J98</f>
-        <v/>
-      </c>
-      <c r="L93" s="85">
-        <f>K98</f>
-        <v/>
-      </c>
-      <c r="M93" s="85">
-        <f>L98</f>
-        <v/>
-      </c>
-      <c r="N93" s="85">
-        <f>M98</f>
-        <v/>
-      </c>
-      <c r="O93" s="85">
-        <f>N98</f>
-        <v/>
-      </c>
-      <c r="P93" s="85">
-        <f>O98</f>
-        <v/>
-      </c>
-      <c r="Q93" s="85">
-        <f>P98</f>
-        <v/>
-      </c>
-      <c r="R93" s="85">
-        <f>D93</f>
-        <v/>
-      </c>
+      <c r="B93" s="65" t="n"/>
+      <c r="C93" s="65" t="n"/>
+      <c r="D93" s="65" t="n"/>
+      <c r="E93" s="65" t="n"/>
+      <c r="F93" s="65" t="n"/>
+      <c r="G93" s="65" t="n"/>
+      <c r="H93" s="65" t="n"/>
+      <c r="I93" s="65" t="n"/>
+      <c r="J93" s="65" t="n"/>
+      <c r="K93" s="65" t="n"/>
+      <c r="L93" s="65" t="n"/>
+      <c r="M93" s="65" t="n"/>
+      <c r="N93" s="65" t="n"/>
+      <c r="O93" s="65" t="n"/>
+      <c r="P93" s="65" t="n"/>
+      <c r="Q93" s="65" t="n"/>
+      <c r="R93" s="65" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   RHB cash deposits</t>
+          <t xml:space="preserve">   RHB opening balance</t>
         </is>
       </c>
       <c r="D94" s="85">
-        <f>D90</f>
+        <f>'Q4 Assumptions'!$B$8</f>
         <v/>
       </c>
       <c r="E94" s="85">
-        <f>E90</f>
+        <f>D99</f>
         <v/>
       </c>
       <c r="F94" s="85">
-        <f>F90</f>
+        <f>E99</f>
         <v/>
       </c>
       <c r="G94" s="85">
-        <f>G90</f>
+        <f>F99</f>
         <v/>
       </c>
       <c r="H94" s="85">
-        <f>H90</f>
+        <f>G99</f>
         <v/>
       </c>
       <c r="I94" s="85">
-        <f>I90</f>
+        <f>H99</f>
         <v/>
       </c>
       <c r="J94" s="85">
-        <f>J90</f>
+        <f>I99</f>
         <v/>
       </c>
       <c r="K94" s="85">
-        <f>K90</f>
+        <f>J99</f>
         <v/>
       </c>
       <c r="L94" s="85">
-        <f>L90</f>
+        <f>K99</f>
         <v/>
       </c>
       <c r="M94" s="85">
-        <f>M90</f>
+        <f>L99</f>
         <v/>
       </c>
       <c r="N94" s="85">
-        <f>N90</f>
+        <f>M99</f>
         <v/>
       </c>
       <c r="O94" s="85">
-        <f>O90</f>
+        <f>N99</f>
         <v/>
       </c>
       <c r="P94" s="85">
-        <f>P90</f>
+        <f>O99</f>
         <v/>
       </c>
       <c r="Q94" s="85">
-        <f>Q90</f>
-        <v/>
-      </c>
-      <c r="R94" s="93">
-        <f>SUM(D94:Q94)</f>
+        <f>P99</f>
+        <v/>
+      </c>
+      <c r="R94" s="85">
+        <f>D94</f>
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   RHB licensing / payroll (incl. +2% per outlet) / bonus</t>
+          <t xml:space="preserve">   RHB cash deposits</t>
         </is>
       </c>
       <c r="D95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)*'Q4 Assumptions'!$B$15*D84</f>
+        <f>D91</f>
         <v/>
       </c>
       <c r="E95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)*'Q4 Assumptions'!$B$15*E84</f>
+        <f>E91</f>
         <v/>
       </c>
       <c r="F95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)*'Q4 Assumptions'!$B$15*F84</f>
+        <f>F91</f>
         <v/>
       </c>
       <c r="G95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)*'Q4 Assumptions'!$B$15*G84</f>
+        <f>G91</f>
         <v/>
       </c>
       <c r="H95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)*'Q4 Assumptions'!$B$15*H84</f>
+        <f>H91</f>
         <v/>
       </c>
       <c r="I95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)*'Q4 Assumptions'!$B$15*I84</f>
+        <f>I91</f>
         <v/>
       </c>
       <c r="J95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)*'Q4 Assumptions'!$B$15*J84</f>
+        <f>J91</f>
         <v/>
       </c>
       <c r="K95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)*'Q4 Assumptions'!$B$15*K84</f>
+        <f>K91</f>
         <v/>
       </c>
       <c r="L95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)*'Q4 Assumptions'!$B$15*L84</f>
+        <f>L91</f>
         <v/>
       </c>
       <c r="M95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)*'Q4 Assumptions'!$B$15*M84</f>
+        <f>M91</f>
         <v/>
       </c>
       <c r="N95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)*'Q4 Assumptions'!$B$15*N84</f>
+        <f>N91</f>
         <v/>
       </c>
       <c r="O95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)*'Q4 Assumptions'!$B$15*O84</f>
+        <f>O91</f>
         <v/>
       </c>
       <c r="P95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)*'Q4 Assumptions'!$B$15*P84</f>
+        <f>P91</f>
         <v/>
       </c>
       <c r="Q95" s="85">
-        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)*'Q4 Assumptions'!$B$15*Q84</f>
+        <f>Q91</f>
         <v/>
       </c>
       <c r="R95" s="93">
@@ -13948,260 +13963,260 @@
     <row r="96">
       <c r="A96" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   RHB balance before top-up</t>
+          <t xml:space="preserve">   RHB licensing / payroll (incl. +2% per outlet) / bonus</t>
         </is>
       </c>
       <c r="D96" s="85">
-        <f>D93+D94+D95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;D$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;D$11)*'Q4 Assumptions'!$B$15*D84</f>
         <v/>
       </c>
       <c r="E96" s="85">
-        <f>E93+E94+E95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;E$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;E$11)*'Q4 Assumptions'!$B$15*E84</f>
         <v/>
       </c>
       <c r="F96" s="85">
-        <f>F93+F94+F95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;F$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;F$11)*'Q4 Assumptions'!$B$15*F84</f>
         <v/>
       </c>
       <c r="G96" s="85">
-        <f>G93+G94+G95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;G$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;G$11)*'Q4 Assumptions'!$B$15*G84</f>
         <v/>
       </c>
       <c r="H96" s="85">
-        <f>H93+H94+H95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;H$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;H$11)*'Q4 Assumptions'!$B$15*H84</f>
         <v/>
       </c>
       <c r="I96" s="85">
-        <f>I93+I94+I95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;I$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;I$11)*'Q4 Assumptions'!$B$15*I84</f>
         <v/>
       </c>
       <c r="J96" s="85">
-        <f>J93+J94+J95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;J$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;J$11)*'Q4 Assumptions'!$B$15*J84</f>
         <v/>
       </c>
       <c r="K96" s="85">
-        <f>K93+K94+K95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;K$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;K$11)*'Q4 Assumptions'!$B$15*K84</f>
         <v/>
       </c>
       <c r="L96" s="85">
-        <f>L93+L94+L95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;L$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;L$11)*'Q4 Assumptions'!$B$15*L84</f>
         <v/>
       </c>
       <c r="M96" s="85">
-        <f>M93+M94+M95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;M$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;M$11)*'Q4 Assumptions'!$B$15*M84</f>
         <v/>
       </c>
       <c r="N96" s="85">
-        <f>N93+N94+N95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;N$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;N$11)*'Q4 Assumptions'!$B$15*N84</f>
         <v/>
       </c>
       <c r="O96" s="85">
-        <f>O93+O94+O95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;O$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;O$11)*'Q4 Assumptions'!$B$15*O84</f>
         <v/>
       </c>
       <c r="P96" s="85">
-        <f>P93+P94+P95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;P$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;P$11)*'Q4 Assumptions'!$B$15*P84</f>
         <v/>
       </c>
       <c r="Q96" s="85">
-        <f>Q93+Q94+Q95</f>
+        <f>SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)+SUMIFS('Q4 Assumptions'!$C$85:$C$133,'Q4 Assumptions'!$E$85:$E$133,"RHB",'Q4 Assumptions'!$F$85:$F$133,"Y",'Q4 Assumptions'!$B$85:$B$133,"&gt;="&amp;Q$10,'Q4 Assumptions'!$B$85:$B$133,"&lt;="&amp;Q$11)*'Q4 Assumptions'!$B$15*Q84</f>
+        <v/>
+      </c>
+      <c r="R96" s="93">
+        <f>SUM(D96:Q96)</f>
         <v/>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="56" t="inlineStr">
         <is>
+          <t xml:space="preserve">   RHB balance before top-up</t>
+        </is>
+      </c>
+      <c r="D97" s="85">
+        <f>D94+D95+D96</f>
+        <v/>
+      </c>
+      <c r="E97" s="85">
+        <f>E94+E95+E96</f>
+        <v/>
+      </c>
+      <c r="F97" s="85">
+        <f>F94+F95+F96</f>
+        <v/>
+      </c>
+      <c r="G97" s="85">
+        <f>G94+G95+G96</f>
+        <v/>
+      </c>
+      <c r="H97" s="85">
+        <f>H94+H95+H96</f>
+        <v/>
+      </c>
+      <c r="I97" s="85">
+        <f>I94+I95+I96</f>
+        <v/>
+      </c>
+      <c r="J97" s="85">
+        <f>J94+J95+J96</f>
+        <v/>
+      </c>
+      <c r="K97" s="85">
+        <f>K94+K95+K96</f>
+        <v/>
+      </c>
+      <c r="L97" s="85">
+        <f>L94+L95+L96</f>
+        <v/>
+      </c>
+      <c r="M97" s="85">
+        <f>M94+M95+M96</f>
+        <v/>
+      </c>
+      <c r="N97" s="85">
+        <f>N94+N95+N96</f>
+        <v/>
+      </c>
+      <c r="O97" s="85">
+        <f>O94+O95+O96</f>
+        <v/>
+      </c>
+      <c r="P97" s="85">
+        <f>P94+P95+P96</f>
+        <v/>
+      </c>
+      <c r="Q97" s="85">
+        <f>Q94+Q95+Q96</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="56" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Transfer Maybank → RHB</t>
         </is>
       </c>
-      <c r="D97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-D96)</f>
-        <v/>
-      </c>
-      <c r="E97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-E96)</f>
-        <v/>
-      </c>
-      <c r="F97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-F96)</f>
-        <v/>
-      </c>
-      <c r="G97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-G96)</f>
-        <v/>
-      </c>
-      <c r="H97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-H96)</f>
-        <v/>
-      </c>
-      <c r="I97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-I96)</f>
-        <v/>
-      </c>
-      <c r="J97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-J96)</f>
-        <v/>
-      </c>
-      <c r="K97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-K96)</f>
-        <v/>
-      </c>
-      <c r="L97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-L96)</f>
-        <v/>
-      </c>
-      <c r="M97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-M96)</f>
-        <v/>
-      </c>
-      <c r="N97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-N96)</f>
-        <v/>
-      </c>
-      <c r="O97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-O96)</f>
-        <v/>
-      </c>
-      <c r="P97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-P96)</f>
-        <v/>
-      </c>
-      <c r="Q97" s="85">
-        <f>MAX(0,'Q4 Assumptions'!$B$29-Q96)</f>
-        <v/>
-      </c>
-      <c r="R97" s="93">
-        <f>SUM(D97:Q97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   RHB closing balance</t>
-        </is>
-      </c>
-      <c r="D98" s="93">
-        <f>D96+D97</f>
-        <v/>
-      </c>
-      <c r="E98" s="93">
-        <f>E96+E97</f>
-        <v/>
-      </c>
-      <c r="F98" s="93">
-        <f>F96+F97</f>
-        <v/>
-      </c>
-      <c r="G98" s="93">
-        <f>G96+G97</f>
-        <v/>
-      </c>
-      <c r="H98" s="93">
-        <f>H96+H97</f>
-        <v/>
-      </c>
-      <c r="I98" s="93">
-        <f>I96+I97</f>
-        <v/>
-      </c>
-      <c r="J98" s="93">
-        <f>J96+J97</f>
-        <v/>
-      </c>
-      <c r="K98" s="93">
-        <f>K96+K97</f>
-        <v/>
-      </c>
-      <c r="L98" s="93">
-        <f>L96+L97</f>
-        <v/>
-      </c>
-      <c r="M98" s="93">
-        <f>M96+M97</f>
-        <v/>
-      </c>
-      <c r="N98" s="93">
-        <f>N96+N97</f>
-        <v/>
-      </c>
-      <c r="O98" s="93">
-        <f>O96+O97</f>
-        <v/>
-      </c>
-      <c r="P98" s="93">
-        <f>P96+P97</f>
-        <v/>
-      </c>
-      <c r="Q98" s="93">
-        <f>Q96+Q97</f>
+      <c r="D98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-D97)</f>
+        <v/>
+      </c>
+      <c r="E98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-E97)</f>
+        <v/>
+      </c>
+      <c r="F98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-F97)</f>
+        <v/>
+      </c>
+      <c r="G98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-G97)</f>
+        <v/>
+      </c>
+      <c r="H98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-H97)</f>
+        <v/>
+      </c>
+      <c r="I98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-I97)</f>
+        <v/>
+      </c>
+      <c r="J98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-J97)</f>
+        <v/>
+      </c>
+      <c r="K98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-K97)</f>
+        <v/>
+      </c>
+      <c r="L98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-L97)</f>
+        <v/>
+      </c>
+      <c r="M98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-M97)</f>
+        <v/>
+      </c>
+      <c r="N98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-N97)</f>
+        <v/>
+      </c>
+      <c r="O98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-O97)</f>
+        <v/>
+      </c>
+      <c r="P98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-P97)</f>
+        <v/>
+      </c>
+      <c r="Q98" s="85">
+        <f>MAX(0,'Q4 Assumptions'!$B$29-Q97)</f>
         <v/>
       </c>
       <c r="R98" s="93">
-        <f>Q98</f>
+        <f>SUM(D98:Q98)</f>
         <v/>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Maybank closing balance</t>
+          <t xml:space="preserve">   RHB closing balance</t>
         </is>
       </c>
       <c r="D99" s="93">
-        <f>D77-D98</f>
+        <f>D97+D98</f>
         <v/>
       </c>
       <c r="E99" s="93">
-        <f>E77-E98</f>
+        <f>E97+E98</f>
         <v/>
       </c>
       <c r="F99" s="93">
-        <f>F77-F98</f>
+        <f>F97+F98</f>
         <v/>
       </c>
       <c r="G99" s="93">
-        <f>G77-G98</f>
+        <f>G97+G98</f>
         <v/>
       </c>
       <c r="H99" s="93">
-        <f>H77-H98</f>
+        <f>H97+H98</f>
         <v/>
       </c>
       <c r="I99" s="93">
-        <f>I77-I98</f>
+        <f>I97+I98</f>
         <v/>
       </c>
       <c r="J99" s="93">
-        <f>J77-J98</f>
+        <f>J97+J98</f>
         <v/>
       </c>
       <c r="K99" s="93">
-        <f>K77-K98</f>
+        <f>K97+K98</f>
         <v/>
       </c>
       <c r="L99" s="93">
-        <f>L77-L98</f>
+        <f>L97+L98</f>
         <v/>
       </c>
       <c r="M99" s="93">
-        <f>M77-M98</f>
+        <f>M97+M98</f>
         <v/>
       </c>
       <c r="N99" s="93">
-        <f>N77-N98</f>
+        <f>N97+N98</f>
         <v/>
       </c>
       <c r="O99" s="93">
-        <f>O77-O98</f>
+        <f>O97+O98</f>
         <v/>
       </c>
       <c r="P99" s="93">
-        <f>P77-P98</f>
+        <f>P97+P98</f>
         <v/>
       </c>
       <c r="Q99" s="93">
-        <f>Q77-Q98</f>
+        <f>Q97+Q98</f>
         <v/>
       </c>
       <c r="R99" s="93">
@@ -14209,13 +14224,80 @@
         <v/>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="52" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Maybank closing balance</t>
+        </is>
+      </c>
+      <c r="D100" s="93">
+        <f>D77-D99</f>
+        <v/>
+      </c>
+      <c r="E100" s="93">
+        <f>E77-E99</f>
+        <v/>
+      </c>
+      <c r="F100" s="93">
+        <f>F77-F99</f>
+        <v/>
+      </c>
+      <c r="G100" s="93">
+        <f>G77-G99</f>
+        <v/>
+      </c>
+      <c r="H100" s="93">
+        <f>H77-H99</f>
+        <v/>
+      </c>
+      <c r="I100" s="93">
+        <f>I77-I99</f>
+        <v/>
+      </c>
+      <c r="J100" s="93">
+        <f>J77-J99</f>
+        <v/>
+      </c>
+      <c r="K100" s="93">
+        <f>K77-K99</f>
+        <v/>
+      </c>
+      <c r="L100" s="93">
+        <f>L77-L99</f>
+        <v/>
+      </c>
+      <c r="M100" s="93">
+        <f>M77-M99</f>
+        <v/>
+      </c>
+      <c r="N100" s="93">
+        <f>N77-N99</f>
+        <v/>
+      </c>
+      <c r="O100" s="93">
+        <f>O77-O99</f>
+        <v/>
+      </c>
+      <c r="P100" s="93">
+        <f>P77-P99</f>
+        <v/>
+      </c>
+      <c r="Q100" s="93">
+        <f>Q77-Q99</f>
+        <v/>
+      </c>
+      <c r="R100" s="93">
+        <f>Q100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="52" t="inlineStr">
         <is>
           <t>Check: Sept'26 column net vs statement −987,655.35 (should be 0)</t>
         </is>
       </c>
-      <c r="C101" s="87">
+      <c r="C102" s="87">
         <f>ROUND(C74-(-987655.35),2)</f>
         <v/>
       </c>

</xml_diff>